<commit_message>
Lock compressed 2018 draft cascade board
</commit_message>
<xml_diff>
--- a/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
+++ b/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R5e9a8a57774e4a37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="Rb4b4a76e845549b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="Rb38bcf29f3f04f21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="4" r:id="R5a854161d79545d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="5" r:id="R6a11b9c68c094133"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="6" r:id="R6f33046343f843bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R243ec70f0c2544d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="R004ae6c0cc164082"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="R89934bb09586473b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R4a11c7dc755f4e8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="5" r:id="Rdfaeae280acc4ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="6" r:id="Ra5b8f023a20e46c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R41ecceb893434cf6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,7 +175,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="60">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -278,6 +279,15 @@
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
@@ -288,12 +298,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
@@ -376,7 +380,26 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SourceTable" displayName="SourceTable" ref="A4:D16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DraftBoardTable" displayName="DraftBoardTable" ref="A6:K37" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="11">
+    <x:tableColumn id="1" name="Pick"/>
+    <x:tableColumn id="2" name="Actual destination"/>
+    <x:tableColumn id="3" name="Actual player"/>
+    <x:tableColumn id="4" name="Actual trade/path"/>
+    <x:tableColumn id="5" name="CF destination"/>
+    <x:tableColumn id="6" name="CF player"/>
+    <x:tableColumn id="7" name="Status"/>
+    <x:tableColumn id="8" name="Incoming displaced"/>
+    <x:tableColumn id="9" name="Decision reason"/>
+    <x:tableColumn id="10" name="Downstream"/>
+    <x:tableColumn id="11" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceTable" displayName="SourceTable" ref="A4:D25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Source"/>
@@ -583,7 +606,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="18" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="36" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="44" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
@@ -594,7 +617,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="18" t="str">
-        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / BASELINE v0.1</x:v>
+        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.2</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -629,7 +652,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>BASELINE_PASS / COUNTERFACTUAL_HOLD</x:v>
+        <x:v>BASELINE_PASS / SECOND_TEAM_IMPACT_HOLD</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
         <x:v>Canon</x:v>
@@ -929,7 +952,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>The 2019 standings/lottery cannot be FINAL until Spellman's new team and that team's season impact are resolved after rerunning 2018 picks 30-60.</x:v>
+        <x:v>Spellman's destination is resolved at San Antonio #49. The 2019 standings/lottery cannot be FINAL until the Spurs' 2018-19 impact is closed.</x:v>
       </x:c>
       <x:c r="C18" s="22"/>
       <x:c r="D18" s="22"/>
@@ -8001,7 +8024,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf909ac086013489a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R187056fa3cab45d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9040,12 +9063,1194 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a13c7de518445bb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4fefc5fb924228"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="16" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="24" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="34" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="24" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="22" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="48" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="28" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="14" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>2018 PICKS 30-60 — COMPRESSED COUNTERFACTUAL BOARD</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="6" t="str">
+        <x:v>Scanned picks</x:v>
+      </x:c>
+      <x:c r="B4" s="6" t="n">
+        <x:f>COUNTA(A7:A37)</x:f>
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C4" s="6" t="str">
+        <x:v>Changed/cascade</x:v>
+      </x:c>
+      <x:c r="D4" s="6" t="n">
+        <x:f>COUNTIF(G7:G37,"CHANGED")+COUNTIF(G7:G37,"CASCADE")</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E4" s="6" t="str">
+        <x:v>Unchanged</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="n">
+        <x:f>COUNTIF(G7:G37,"UNCHANGED")</x:f>
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="G4" s="6" t="str">
+        <x:v>Next blocker</x:v>
+      </x:c>
+      <x:c r="H4" s="6" t="str">
+        <x:v>Spurs 2018-19 impact</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="11" t="str">
+        <x:v>Pick</x:v>
+      </x:c>
+      <x:c r="B6" s="11" t="str">
+        <x:v>Actual destination</x:v>
+      </x:c>
+      <x:c r="C6" s="11" t="str">
+        <x:v>Actual player</x:v>
+      </x:c>
+      <x:c r="D6" s="11" t="str">
+        <x:v>Actual trade/path</x:v>
+      </x:c>
+      <x:c r="E6" s="11" t="str">
+        <x:v>CF destination</x:v>
+      </x:c>
+      <x:c r="F6" s="11" t="str">
+        <x:v>CF player</x:v>
+      </x:c>
+      <x:c r="G6" s="11" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="H6" s="11" t="str">
+        <x:v>Incoming displaced</x:v>
+      </x:c>
+      <x:c r="I6" s="11" t="str">
+        <x:v>Decision reason</x:v>
+      </x:c>
+      <x:c r="J6" s="11" t="str">
+        <x:v>Downstream</x:v>
+      </x:c>
+      <x:c r="K6" s="11" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="53" t="n">
+        <x:v>30</x:v>
+      </x:c>
+      <x:c r="B7" s="53" t="str">
+        <x:v>Atlanta Hawks</x:v>
+      </x:c>
+      <x:c r="C7" s="53" t="str">
+        <x:v>Omari Spellman</x:v>
+      </x:c>
+      <x:c r="D7" s="53" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E7" s="53" t="str">
+        <x:v>Atlanta Hawks</x:v>
+      </x:c>
+      <x:c r="F7" s="53" t="str">
+        <x:v>Fictional protagonist</x:v>
+      </x:c>
+      <x:c r="G7" s="53" t="str">
+        <x:v>CHANGED</x:v>
+      </x:c>
+      <x:c r="H7" s="53" t="str">
+        <x:v>Protagonist</x:v>
+      </x:c>
+      <x:c r="I7" s="53" t="str">
+        <x:v>The new player occupies Atlanta's actual #30 slot.</x:v>
+      </x:c>
+      <x:c r="J7" s="53" t="str">
+        <x:v>Atlanta roster/minutes rerun</x:v>
+      </x:c>
+      <x:c r="K7" s="53" t="str">
+        <x:v>S12/S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="51" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="B8" s="51" t="str">
+        <x:v>Phoenix Suns</x:v>
+      </x:c>
+      <x:c r="C8" s="51" t="str">
+        <x:v>Elie Okobo</x:v>
+      </x:c>
+      <x:c r="D8" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E8" s="51" t="str">
+        <x:v>Phoenix Suns</x:v>
+      </x:c>
+      <x:c r="F8" s="51" t="str">
+        <x:v>Elie Okobo</x:v>
+      </x:c>
+      <x:c r="G8" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H8" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I8" s="51" t="str">
+        <x:v>Guard-development choice remains rational.</x:v>
+      </x:c>
+      <x:c r="J8" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K8" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="51" t="n">
+        <x:v>32</x:v>
+      </x:c>
+      <x:c r="B9" s="51" t="str">
+        <x:v>Memphis Grizzlies</x:v>
+      </x:c>
+      <x:c r="C9" s="51" t="str">
+        <x:v>Jevon Carter</x:v>
+      </x:c>
+      <x:c r="D9" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E9" s="51" t="str">
+        <x:v>Memphis Grizzlies</x:v>
+      </x:c>
+      <x:c r="F9" s="51" t="str">
+        <x:v>Jevon Carter</x:v>
+      </x:c>
+      <x:c r="G9" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H9" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I9" s="51" t="str">
+        <x:v>Point-of-attack guard need remains distinct.</x:v>
+      </x:c>
+      <x:c r="J9" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K9" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="51" t="n">
+        <x:v>33</x:v>
+      </x:c>
+      <x:c r="B10" s="51" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="C10" s="51" t="str">
+        <x:v>Jalen Brunson</x:v>
+      </x:c>
+      <x:c r="D10" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E10" s="51" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="F10" s="51" t="str">
+        <x:v>Jalen Brunson</x:v>
+      </x:c>
+      <x:c r="G10" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H10" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I10" s="51" t="str">
+        <x:v>Lead-guard depth remains the stronger fit.</x:v>
+      </x:c>
+      <x:c r="J10" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K10" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="51" t="n">
+        <x:v>34</x:v>
+      </x:c>
+      <x:c r="B11" s="51" t="str">
+        <x:v>Charlotte Hornets</x:v>
+      </x:c>
+      <x:c r="C11" s="51" t="str">
+        <x:v>Devonte' Graham</x:v>
+      </x:c>
+      <x:c r="D11" s="51" t="str">
+        <x:v>Rights from ATL for 2019 + 2023 seconds</x:v>
+      </x:c>
+      <x:c r="E11" s="51" t="str">
+        <x:v>Charlotte Hornets</x:v>
+      </x:c>
+      <x:c r="F11" s="51" t="str">
+        <x:v>Devonte' Graham</x:v>
+      </x:c>
+      <x:c r="G11" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H11" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I11" s="51" t="str">
+        <x:v>Charlotte paid two future seconds for a directed guard choice.</x:v>
+      </x:c>
+      <x:c r="J11" s="51" t="str">
+        <x:v>ATL asset trade preserved</x:v>
+      </x:c>
+      <x:c r="K11" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="51" t="n">
+        <x:v>35</x:v>
+      </x:c>
+      <x:c r="B12" s="51" t="str">
+        <x:v>Orlando Magic</x:v>
+      </x:c>
+      <x:c r="C12" s="51" t="str">
+        <x:v>Melvin Frazier</x:v>
+      </x:c>
+      <x:c r="D12" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E12" s="51" t="str">
+        <x:v>Orlando Magic</x:v>
+      </x:c>
+      <x:c r="F12" s="51" t="str">
+        <x:v>Melvin Frazier</x:v>
+      </x:c>
+      <x:c r="G12" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H12" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I12" s="51" t="str">
+        <x:v>Wing-development lane remains distinct.</x:v>
+      </x:c>
+      <x:c r="J12" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K12" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="51" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B13" s="51" t="str">
+        <x:v>New York Knicks</x:v>
+      </x:c>
+      <x:c r="C13" s="51" t="str">
+        <x:v>Mitchell Robinson</x:v>
+      </x:c>
+      <x:c r="D13" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E13" s="51" t="str">
+        <x:v>New York Knicks</x:v>
+      </x:c>
+      <x:c r="F13" s="51" t="str">
+        <x:v>Mitchell Robinson</x:v>
+      </x:c>
+      <x:c r="G13" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H13" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I13" s="51" t="str">
+        <x:v>Robinson's upside remains the board priority.</x:v>
+      </x:c>
+      <x:c r="J13" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K13" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="51" t="n">
+        <x:v>37</x:v>
+      </x:c>
+      <x:c r="B14" s="51" t="str">
+        <x:v>Portland Trail Blazers</x:v>
+      </x:c>
+      <x:c r="C14" s="51" t="str">
+        <x:v>Gary Trent Jr.</x:v>
+      </x:c>
+      <x:c r="D14" s="51" t="str">
+        <x:v>Rights from SAC</x:v>
+      </x:c>
+      <x:c r="E14" s="51" t="str">
+        <x:v>Portland Trail Blazers</x:v>
+      </x:c>
+      <x:c r="F14" s="51" t="str">
+        <x:v>Gary Trent Jr.</x:v>
+      </x:c>
+      <x:c r="G14" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H14" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I14" s="51" t="str">
+        <x:v>Perimeter shooting/development need remains.</x:v>
+      </x:c>
+      <x:c r="J14" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K14" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="51" t="n">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="B15" s="51" t="str">
+        <x:v>Detroit Pistons</x:v>
+      </x:c>
+      <x:c r="C15" s="51" t="str">
+        <x:v>Khyri Thomas</x:v>
+      </x:c>
+      <x:c r="D15" s="51" t="str">
+        <x:v>Rights from PHI</x:v>
+      </x:c>
+      <x:c r="E15" s="51" t="str">
+        <x:v>Detroit Pistons</x:v>
+      </x:c>
+      <x:c r="F15" s="51" t="str">
+        <x:v>Khyri Thomas</x:v>
+      </x:c>
+      <x:c r="G15" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H15" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I15" s="51" t="str">
+        <x:v>Perimeter defense need remains distinct.</x:v>
+      </x:c>
+      <x:c r="J15" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K15" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="51" t="n">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="B16" s="51" t="str">
+        <x:v>Los Angeles Lakers</x:v>
+      </x:c>
+      <x:c r="C16" s="51" t="str">
+        <x:v>Isaac Bonga</x:v>
+      </x:c>
+      <x:c r="D16" s="51" t="str">
+        <x:v>Rights from PHI</x:v>
+      </x:c>
+      <x:c r="E16" s="51" t="str">
+        <x:v>Los Angeles Lakers</x:v>
+      </x:c>
+      <x:c r="F16" s="51" t="str">
+        <x:v>Isaac Bonga</x:v>
+      </x:c>
+      <x:c r="G16" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H16" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I16" s="51" t="str">
+        <x:v>Lakers already used #25 on stretch big Moritz Wagner.</x:v>
+      </x:c>
+      <x:c r="J16" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K16" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="51" t="n">
+        <x:v>40</x:v>
+      </x:c>
+      <x:c r="B17" s="51" t="str">
+        <x:v>Brooklyn Nets</x:v>
+      </x:c>
+      <x:c r="C17" s="51" t="str">
+        <x:v>Rodions Kurucs</x:v>
+      </x:c>
+      <x:c r="D17" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E17" s="51" t="str">
+        <x:v>Brooklyn Nets</x:v>
+      </x:c>
+      <x:c r="F17" s="51" t="str">
+        <x:v>Rodions Kurucs</x:v>
+      </x:c>
+      <x:c r="G17" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H17" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I17" s="51" t="str">
+        <x:v>Long-running Kurucs scouting interest remains decisive.</x:v>
+      </x:c>
+      <x:c r="J17" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K17" s="51" t="str">
+        <x:v>S17</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="51" t="n">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="B18" s="51" t="str">
+        <x:v>Denver Nuggets</x:v>
+      </x:c>
+      <x:c r="C18" s="51" t="str">
+        <x:v>Jarred Vanderbilt</x:v>
+      </x:c>
+      <x:c r="D18" s="51" t="str">
+        <x:v>Rights from ORL</x:v>
+      </x:c>
+      <x:c r="E18" s="51" t="str">
+        <x:v>Denver Nuggets</x:v>
+      </x:c>
+      <x:c r="F18" s="51" t="str">
+        <x:v>Jarred Vanderbilt</x:v>
+      </x:c>
+      <x:c r="G18" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H18" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I18" s="51" t="str">
+        <x:v>Vanderbilt upside remains the preferred development bet.</x:v>
+      </x:c>
+      <x:c r="J18" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K18" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="51" t="n">
+        <x:v>42</x:v>
+      </x:c>
+      <x:c r="B19" s="51" t="str">
+        <x:v>Detroit Pistons</x:v>
+      </x:c>
+      <x:c r="C19" s="51" t="str">
+        <x:v>Bruce Brown</x:v>
+      </x:c>
+      <x:c r="D19" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E19" s="51" t="str">
+        <x:v>Detroit Pistons</x:v>
+      </x:c>
+      <x:c r="F19" s="51" t="str">
+        <x:v>Bruce Brown</x:v>
+      </x:c>
+      <x:c r="G19" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H19" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I19" s="51" t="str">
+        <x:v>Guard/wing role remains distinct.</x:v>
+      </x:c>
+      <x:c r="J19" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K19" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="51" t="n">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="B20" s="51" t="str">
+        <x:v>Orlando Magic</x:v>
+      </x:c>
+      <x:c r="C20" s="51" t="str">
+        <x:v>Justin Jackson</x:v>
+      </x:c>
+      <x:c r="D20" s="51" t="str">
+        <x:v>Rights from DEN</x:v>
+      </x:c>
+      <x:c r="E20" s="51" t="str">
+        <x:v>Orlando Magic</x:v>
+      </x:c>
+      <x:c r="F20" s="51" t="str">
+        <x:v>Justin Jackson</x:v>
+      </x:c>
+      <x:c r="G20" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H20" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I20" s="51" t="str">
+        <x:v>Wing-development lane remains distinct.</x:v>
+      </x:c>
+      <x:c r="J20" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K20" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="51" t="n">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="B21" s="51" t="str">
+        <x:v>Washington Wizards</x:v>
+      </x:c>
+      <x:c r="C21" s="51" t="str">
+        <x:v>Issuf Sanon</x:v>
+      </x:c>
+      <x:c r="D21" s="51" t="str">
+        <x:v>Own pick; overseas stash</x:v>
+      </x:c>
+      <x:c r="E21" s="51" t="str">
+        <x:v>Washington Wizards</x:v>
+      </x:c>
+      <x:c r="F21" s="51" t="str">
+        <x:v>Issuf Sanon</x:v>
+      </x:c>
+      <x:c r="G21" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H21" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I21" s="51" t="str">
+        <x:v>Roster/cap plan explicitly favored an overseas stash.</x:v>
+      </x:c>
+      <x:c r="J21" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K21" s="51" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="51" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="B22" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="C22" s="51" t="str">
+        <x:v>Hamidou Diallo</x:v>
+      </x:c>
+      <x:c r="D22" s="51" t="str">
+        <x:v>Rights via BKN/CHA</x:v>
+      </x:c>
+      <x:c r="E22" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="F22" s="51" t="str">
+        <x:v>Hamidou Diallo</x:v>
+      </x:c>
+      <x:c r="G22" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H22" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I22" s="51" t="str">
+        <x:v>Athletic guard target remains distinct.</x:v>
+      </x:c>
+      <x:c r="J22" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K22" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="51" t="n">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="B23" s="51" t="str">
+        <x:v>Houston Rockets</x:v>
+      </x:c>
+      <x:c r="C23" s="51" t="str">
+        <x:v>De'Anthony Melton</x:v>
+      </x:c>
+      <x:c r="D23" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E23" s="51" t="str">
+        <x:v>Houston Rockets</x:v>
+      </x:c>
+      <x:c r="F23" s="51" t="str">
+        <x:v>De'Anthony Melton</x:v>
+      </x:c>
+      <x:c r="G23" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H23" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I23" s="51" t="str">
+        <x:v>Guard asset profile remains distinct.</x:v>
+      </x:c>
+      <x:c r="J23" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K23" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="51" t="n">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="B24" s="51" t="str">
+        <x:v>Los Angeles Lakers</x:v>
+      </x:c>
+      <x:c r="C24" s="51" t="str">
+        <x:v>Svi Mykhailiuk</x:v>
+      </x:c>
+      <x:c r="D24" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E24" s="51" t="str">
+        <x:v>Los Angeles Lakers</x:v>
+      </x:c>
+      <x:c r="F24" s="51" t="str">
+        <x:v>Svi Mykhailiuk</x:v>
+      </x:c>
+      <x:c r="G24" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H24" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I24" s="51" t="str">
+        <x:v>Shooting role remains distinct.</x:v>
+      </x:c>
+      <x:c r="J24" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K24" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="51" t="n">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="B25" s="51" t="str">
+        <x:v>Minnesota Timberwolves</x:v>
+      </x:c>
+      <x:c r="C25" s="51" t="str">
+        <x:v>Keita Bates-Diop</x:v>
+      </x:c>
+      <x:c r="D25" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E25" s="51" t="str">
+        <x:v>Minnesota Timberwolves</x:v>
+      </x:c>
+      <x:c r="F25" s="51" t="str">
+        <x:v>Keita Bates-Diop</x:v>
+      </x:c>
+      <x:c r="G25" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H25" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I25" s="51" t="str">
+        <x:v>Wing-forward choice does not require a cascade.</x:v>
+      </x:c>
+      <x:c r="J25" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K25" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="53" t="n">
+        <x:v>49</x:v>
+      </x:c>
+      <x:c r="B26" s="53" t="str">
+        <x:v>San Antonio Spurs</x:v>
+      </x:c>
+      <x:c r="C26" s="53" t="str">
+        <x:v>Chimezie Metu</x:v>
+      </x:c>
+      <x:c r="D26" s="53" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E26" s="53" t="str">
+        <x:v>San Antonio Spurs</x:v>
+      </x:c>
+      <x:c r="F26" s="53" t="str">
+        <x:v>Omari Spellman</x:v>
+      </x:c>
+      <x:c r="G26" s="53" t="str">
+        <x:v>CHANGED</x:v>
+      </x:c>
+      <x:c r="H26" s="53" t="str">
+        <x:v>Spellman</x:v>
+      </x:c>
+      <x:c r="I26" s="53" t="str">
+        <x:v>Spellman worked out for San Antonio and fit its spacing/IQ profile.</x:v>
+      </x:c>
+      <x:c r="J26" s="53" t="str">
+        <x:v>Spurs 2018-19 impact HOLD</x:v>
+      </x:c>
+      <x:c r="K26" s="53" t="str">
+        <x:v>S14/S15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="51" t="n">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="B27" s="51" t="str">
+        <x:v>Indiana Pacers</x:v>
+      </x:c>
+      <x:c r="C27" s="51" t="str">
+        <x:v>Alize Johnson</x:v>
+      </x:c>
+      <x:c r="D27" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E27" s="51" t="str">
+        <x:v>Indiana Pacers</x:v>
+      </x:c>
+      <x:c r="F27" s="51" t="str">
+        <x:v>Alize Johnson</x:v>
+      </x:c>
+      <x:c r="G27" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H27" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I27" s="51" t="str">
+        <x:v>Actual forward choice remains available.</x:v>
+      </x:c>
+      <x:c r="J27" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K27" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="51" t="n">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="B28" s="51" t="str">
+        <x:v>New Orleans Pelicans</x:v>
+      </x:c>
+      <x:c r="C28" s="51" t="str">
+        <x:v>Tony Carr</x:v>
+      </x:c>
+      <x:c r="D28" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E28" s="51" t="str">
+        <x:v>New Orleans Pelicans</x:v>
+      </x:c>
+      <x:c r="F28" s="51" t="str">
+        <x:v>Tony Carr</x:v>
+      </x:c>
+      <x:c r="G28" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H28" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I28" s="51" t="str">
+        <x:v>Guard-development choice remains distinct.</x:v>
+      </x:c>
+      <x:c r="J28" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K28" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="51" t="n">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="B29" s="51" t="str">
+        <x:v>Houston Rockets</x:v>
+      </x:c>
+      <x:c r="C29" s="51" t="str">
+        <x:v>Vincent Edwards</x:v>
+      </x:c>
+      <x:c r="D29" s="51" t="str">
+        <x:v>Rights from UTA</x:v>
+      </x:c>
+      <x:c r="E29" s="51" t="str">
+        <x:v>Houston Rockets</x:v>
+      </x:c>
+      <x:c r="F29" s="51" t="str">
+        <x:v>Vincent Edwards</x:v>
+      </x:c>
+      <x:c r="G29" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H29" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I29" s="51" t="str">
+        <x:v>Wing-development choice remains distinct.</x:v>
+      </x:c>
+      <x:c r="J29" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K29" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="51" t="n">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="B30" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="C30" s="51" t="str">
+        <x:v>Devon Hall</x:v>
+      </x:c>
+      <x:c r="D30" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E30" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="F30" s="51" t="str">
+        <x:v>Devon Hall</x:v>
+      </x:c>
+      <x:c r="G30" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H30" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I30" s="51" t="str">
+        <x:v>Perimeter/stash route remains distinct.</x:v>
+      </x:c>
+      <x:c r="J30" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K30" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="51" t="n">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="B31" s="51" t="str">
+        <x:v>Philadelphia 76ers</x:v>
+      </x:c>
+      <x:c r="C31" s="51" t="str">
+        <x:v>Shake Milton</x:v>
+      </x:c>
+      <x:c r="D31" s="51" t="str">
+        <x:v>Rights from DAL</x:v>
+      </x:c>
+      <x:c r="E31" s="51" t="str">
+        <x:v>Philadelphia 76ers</x:v>
+      </x:c>
+      <x:c r="F31" s="51" t="str">
+        <x:v>Shake Milton</x:v>
+      </x:c>
+      <x:c r="G31" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H31" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I31" s="51" t="str">
+        <x:v>Guard target and trade structure remain intact.</x:v>
+      </x:c>
+      <x:c r="J31" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K31" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="51" t="n">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="B32" s="51" t="str">
+        <x:v>Charlotte Hornets</x:v>
+      </x:c>
+      <x:c r="C32" s="51" t="str">
+        <x:v>Arnoldas Kulboka</x:v>
+      </x:c>
+      <x:c r="D32" s="51" t="str">
+        <x:v>Own pick; overseas stash</x:v>
+      </x:c>
+      <x:c r="E32" s="51" t="str">
+        <x:v>Charlotte Hornets</x:v>
+      </x:c>
+      <x:c r="F32" s="51" t="str">
+        <x:v>Arnoldas Kulboka</x:v>
+      </x:c>
+      <x:c r="G32" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H32" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I32" s="51" t="str">
+        <x:v>Overseas-stash route remains distinct.</x:v>
+      </x:c>
+      <x:c r="J32" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K32" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="53" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="B33" s="53" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="C33" s="53" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="D33" s="53" t="str">
+        <x:v>Rights from PHI</x:v>
+      </x:c>
+      <x:c r="E33" s="53" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="F33" s="53" t="str">
+        <x:v>Chimezie Metu</x:v>
+      </x:c>
+      <x:c r="G33" s="53" t="str">
+        <x:v>CASCADE</x:v>
+      </x:c>
+      <x:c r="H33" s="53" t="str">
+        <x:v>Metu</x:v>
+      </x:c>
+      <x:c r="I33" s="53" t="str">
+        <x:v>Metu is the displaced #49 athletic big and remains above this slot.</x:v>
+      </x:c>
+      <x:c r="J33" s="53" t="str">
+        <x:v>Dallas role/minutes HOLD</x:v>
+      </x:c>
+      <x:c r="K33" s="53" t="str">
+        <x:v>S13/S15</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="51" t="n">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="B34" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="C34" s="51" t="str">
+        <x:v>Kevin Hervey</x:v>
+      </x:c>
+      <x:c r="D34" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E34" s="51" t="str">
+        <x:v>Oklahoma City Thunder</x:v>
+      </x:c>
+      <x:c r="F34" s="51" t="str">
+        <x:v>Kevin Hervey</x:v>
+      </x:c>
+      <x:c r="G34" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H34" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I34" s="51" t="str">
+        <x:v>Actual forward choice remains available.</x:v>
+      </x:c>
+      <x:c r="J34" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K34" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="53" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="B35" s="53" t="str">
+        <x:v>Denver Nuggets</x:v>
+      </x:c>
+      <x:c r="C35" s="53" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="D35" s="53" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E35" s="53" t="str">
+        <x:v>Denver Nuggets</x:v>
+      </x:c>
+      <x:c r="F35" s="53" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="G35" s="53" t="str">
+        <x:v>CASCADE</x:v>
+      </x:c>
+      <x:c r="H35" s="53" t="str">
+        <x:v>Spalding</x:v>
+      </x:c>
+      <x:c r="I35" s="53" t="str">
+        <x:v>Spalding was graded in the drafted second-round big tier.</x:v>
+      </x:c>
+      <x:c r="J35" s="53" t="str">
+        <x:v>Denver role/two-way HOLD</x:v>
+      </x:c>
+      <x:c r="K35" s="53" t="str">
+        <x:v>S18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="51" t="n">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="B36" s="51" t="str">
+        <x:v>Phoenix Suns</x:v>
+      </x:c>
+      <x:c r="C36" s="51" t="str">
+        <x:v>George King</x:v>
+      </x:c>
+      <x:c r="D36" s="51" t="str">
+        <x:v>Own pick</x:v>
+      </x:c>
+      <x:c r="E36" s="51" t="str">
+        <x:v>Phoenix Suns</x:v>
+      </x:c>
+      <x:c r="F36" s="51" t="str">
+        <x:v>George King</x:v>
+      </x:c>
+      <x:c r="G36" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H36" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I36" s="51" t="str">
+        <x:v>Actual wing choice remains available.</x:v>
+      </x:c>
+      <x:c r="J36" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K36" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="51" t="n">
+        <x:v>60</x:v>
+      </x:c>
+      <x:c r="B37" s="51" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="C37" s="51" t="str">
+        <x:v>Kostas Antetokounmpo</x:v>
+      </x:c>
+      <x:c r="D37" s="51" t="str">
+        <x:v>Rights from PHI</x:v>
+      </x:c>
+      <x:c r="E37" s="51" t="str">
+        <x:v>Dallas Mavericks</x:v>
+      </x:c>
+      <x:c r="F37" s="51" t="str">
+        <x:v>Kostas Antetokounmpo</x:v>
+      </x:c>
+      <x:c r="G37" s="52" t="str">
+        <x:v>UNCHANGED</x:v>
+      </x:c>
+      <x:c r="H37" s="51" t="str">
+        <x:v>None</x:v>
+      </x:c>
+      <x:c r="I37" s="51" t="str">
+        <x:v>Second acquired pick and upside bet remain intact.</x:v>
+      </x:c>
+      <x:c r="J37" s="51" t="str">
+        <x:v>Actual path preserved</x:v>
+      </x:c>
+      <x:c r="K37" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:K2"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd845085108c84979"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9111,10 +10316,10 @@
       <x:c r="D5" s="13" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="51" t="n">
+      <x:c r="E5" s="54" t="n">
         <x:v>0.105</x:v>
       </x:c>
-      <x:c r="F5" s="51" t="n">
+      <x:c r="F5" s="54" t="n">
         <x:v>0.4212</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
@@ -9143,10 +10348,10 @@
       <x:c r="D6" s="13" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E6" s="51" t="n">
+      <x:c r="E6" s="54" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="F6" s="51" t="n">
+      <x:c r="F6" s="54" t="n">
         <x:v>0.263</x:v>
       </x:c>
       <x:c r="G6" s="13" t="n">
@@ -9242,8 +10447,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="54" t="str">
-        <x:v>FINAL BLOCKER: rerun the 2018 #30-60 board, resolve Spellman's new team, and close that team's 2018-19 impact.</x:v>
+      <x:c r="A14" s="57" t="str">
+        <x:v>FINAL BLOCKER: Spellman is resolved to San Antonio #49; close the Spurs' 2018-19 rotation and game impact before standings/lottery.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9257,7 +10462,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9295,225 +10500,225 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="56" t="str">
+      <x:c r="A5" s="51" t="str">
         <x:v>G0</x:v>
       </x:c>
-      <x:c r="B5" s="56" t="str">
+      <x:c r="B5" s="51" t="str">
         <x:v>Spellman destination + second-team impact</x:v>
       </x:c>
-      <x:c r="C5" s="56" t="str">
-        <x:v>Unresolved after 2018 #30</x:v>
-      </x:c>
-      <x:c r="D5" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E5" s="56" t="str">
+      <x:c r="C5" s="51" t="str">
+        <x:v>Spellman → Spurs #49; Spurs impact not executed</x:v>
+      </x:c>
+      <x:c r="D5" s="53" t="str">
+        <x:v>PARTIAL</x:v>
+      </x:c>
+      <x:c r="E5" s="51" t="str">
         <x:v>FINAL standings/lottery</x:v>
       </x:c>
-      <x:c r="F5" s="56" t="str">
-        <x:v>Run 2018 picks 30-60</x:v>
+      <x:c r="F5" s="51" t="str">
+        <x:v>Model Spurs 2018-19</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="56" t="str">
+      <x:c r="A6" s="51" t="str">
         <x:v>G1</x:v>
       </x:c>
-      <x:c r="B6" s="56" t="str">
+      <x:c r="B6" s="51" t="str">
         <x:v>82 unique + 29-53 + score/OT checksum</x:v>
       </x:c>
-      <x:c r="C6" s="56" t="str">
+      <x:c r="C6" s="51" t="str">
         <x:v>82 rows; 29-53; 9,294 pts; 19,855 game-min</x:v>
       </x:c>
-      <x:c r="D6" s="57" t="str">
+      <x:c r="D6" s="53" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="E6" s="56" t="str">
+      <x:c r="E6" s="51" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="F6" s="56" t="str">
+      <x:c r="F6" s="51" t="str">
         <x:v>Preserve immutable baseline</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="56" t="str">
+      <x:c r="A7" s="51" t="str">
         <x:v>G2</x:v>
       </x:c>
-      <x:c r="B7" s="56" t="str">
+      <x:c r="B7" s="51" t="str">
         <x:v>Rotation/assignment/impact priors before results</x:v>
       </x:c>
-      <x:c r="C7" s="56" t="str">
+      <x:c r="C7" s="51" t="str">
         <x:v>Only season range locked</x:v>
       </x:c>
-      <x:c r="D7" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E7" s="56" t="str">
+      <x:c r="D7" s="53" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="E7" s="51" t="str">
         <x:v>CF execution</x:v>
       </x:c>
-      <x:c r="F7" s="56" t="str">
+      <x:c r="F7" s="51" t="str">
         <x:v>Build date-specific availability</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="56" t="str">
+      <x:c r="A8" s="51" t="str">
         <x:v>G3</x:v>
       </x:c>
-      <x:c r="B8" s="56" t="str">
+      <x:c r="B8" s="51" t="str">
         <x:v>Every game minute-conserved; no NBA/Erie collision</x:v>
       </x:c>
-      <x:c r="C8" s="56" t="str">
+      <x:c r="C8" s="51" t="str">
         <x:v>Season cap proven; player-game not built</x:v>
       </x:c>
-      <x:c r="D8" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E8" s="56" t="str">
+      <x:c r="D8" s="53" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="E8" s="51" t="str">
         <x:v>CF execution</x:v>
       </x:c>
-      <x:c r="F8" s="56" t="str">
+      <x:c r="F8" s="51" t="str">
         <x:v>Create player-game donor vectors</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="56" t="str">
+      <x:c r="A9" s="51" t="str">
         <x:v>G4</x:v>
       </x:c>
-      <x:c r="B9" s="56" t="str">
+      <x:c r="B9" s="51" t="str">
         <x:v>All 82 games contact classified</x:v>
       </x:c>
-      <x:c r="C9" s="56" t="str">
+      <x:c r="C9" s="51" t="str">
         <x:v>82/82 ROSTER</x:v>
       </x:c>
-      <x:c r="D9" s="57" t="str">
+      <x:c r="D9" s="53" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="E9" s="56" t="str">
+      <x:c r="E9" s="51" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="F9" s="56" t="str">
+      <x:c r="F9" s="51" t="str">
         <x:v>Upgrade DIRECT/CASCADE as needed</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="56" t="str">
+      <x:c r="A10" s="51" t="str">
         <x:v>G5</x:v>
       </x:c>
-      <x:c r="B10" s="56" t="str">
+      <x:c r="B10" s="51" t="str">
         <x:v>Pregame-only pB; fixed latent u; no manual flip</x:v>
       </x:c>
-      <x:c r="C10" s="56" t="str">
+      <x:c r="C10" s="51" t="str">
         <x:v>Method selected; inputs absent</x:v>
       </x:c>
-      <x:c r="D10" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E10" s="56" t="str">
+      <x:c r="D10" s="53" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="E10" s="51" t="str">
         <x:v>CF result</x:v>
       </x:c>
-      <x:c r="F10" s="56" t="str">
+      <x:c r="F10" s="51" t="str">
         <x:v>Calibrate and preregister</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="56" t="str">
+      <x:c r="A11" s="51" t="str">
         <x:v>G6</x:v>
       </x:c>
-      <x:c r="B11" s="56" t="str">
+      <x:c r="B11" s="51" t="str">
         <x:v>Chronological injury/fatigue/trade updates</x:v>
       </x:c>
-      <x:c r="C11" s="56" t="str">
+      <x:c r="C11" s="51" t="str">
         <x:v>Not executed</x:v>
       </x:c>
-      <x:c r="D11" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E11" s="56" t="str">
+      <x:c r="D11" s="53" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="E11" s="51" t="str">
         <x:v>CF result</x:v>
       </x:c>
-      <x:c r="F11" s="56" t="str">
+      <x:c r="F11" s="51" t="str">
         <x:v>Process in date order</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="56" t="str">
+      <x:c r="A12" s="51" t="str">
         <x:v>G7</x:v>
       </x:c>
-      <x:c r="B12" s="56" t="str">
+      <x:c r="B12" s="51" t="str">
         <x:v>No exact score invention; sensitivity isolated</x:v>
       </x:c>
-      <x:c r="C12" s="56" t="str">
+      <x:c r="C12" s="51" t="str">
         <x:v>No CF scores/results created</x:v>
       </x:c>
-      <x:c r="D12" s="57" t="str">
+      <x:c r="D12" s="53" t="str">
         <x:v>PASS</x:v>
       </x:c>
-      <x:c r="E12" s="56" t="str">
+      <x:c r="E12" s="51" t="str">
         <x:v>None</x:v>
       </x:c>
-      <x:c r="F12" s="56" t="str">
+      <x:c r="F12" s="51" t="str">
         <x:v>Keep results HOLD until model</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="56" t="str">
+      <x:c r="A13" s="51" t="str">
         <x:v>G8</x:v>
       </x:c>
-      <x:c r="B13" s="56" t="str">
+      <x:c r="B13" s="51" t="str">
         <x:v>Opponent W/L + league standings/tiebreaker</x:v>
       </x:c>
-      <x:c r="C13" s="56" t="str">
+      <x:c r="C13" s="51" t="str">
         <x:v>Not executed</x:v>
       </x:c>
-      <x:c r="D13" s="57" t="str">
-        <x:v>HOLD</x:v>
-      </x:c>
-      <x:c r="E13" s="56" t="str">
+      <x:c r="D13" s="53" t="str">
+        <x:v>HOLD</x:v>
+      </x:c>
+      <x:c r="E13" s="51" t="str">
         <x:v>2019 lottery</x:v>
       </x:c>
-      <x:c r="F13" s="56" t="str">
+      <x:c r="F13" s="51" t="str">
         <x:v>Build league bridge</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="56" t="str">
+      <x:c r="A14" s="51" t="str">
         <x:v>G9</x:v>
       </x:c>
-      <x:c r="B14" s="56" t="str">
+      <x:c r="B14" s="51" t="str">
         <x:v>Raw baseline immutable; run/model/seed logged</x:v>
       </x:c>
-      <x:c r="C14" s="56" t="str">
+      <x:c r="C14" s="51" t="str">
         <x:v>Workbook baseline created</x:v>
       </x:c>
-      <x:c r="D14" s="57" t="str">
+      <x:c r="D14" s="53" t="str">
         <x:v>PARTIAL</x:v>
       </x:c>
-      <x:c r="E14" s="56" t="str">
+      <x:c r="E14" s="51" t="str">
         <x:v>Reproduction</x:v>
       </x:c>
-      <x:c r="F14" s="56" t="str">
+      <x:c r="F14" s="51" t="str">
         <x:v>Add run manifest after preregistration</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="58"/>
-      <x:c r="B15" s="58"/>
-      <x:c r="C15" s="58"/>
-      <x:c r="D15" s="58"/>
-      <x:c r="E15" s="58"/>
-      <x:c r="F15" s="58"/>
+      <x:c r="A15" s="59"/>
+      <x:c r="B15" s="59"/>
+      <x:c r="C15" s="59"/>
+      <x:c r="D15" s="59"/>
+      <x:c r="E15" s="59"/>
+      <x:c r="F15" s="59"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="50" t="str">
         <x:v>OVERALL</x:v>
       </x:c>
       <x:c r="B16" s="50" t="str">
-        <x:v>BASELINE_PASS / COUNTERFACTUAL_HOLD</x:v>
+        <x:v>BASELINE_PASS / SECOND_TEAM_IMPACT_HOLD</x:v>
       </x:c>
       <x:c r="C16" s="50"/>
       <x:c r="D16" s="50"/>
       <x:c r="E16" s="50"/>
       <x:c r="F16" s="50" t="str">
-        <x:v>Atlanta-local PROVISIONAL_PASS not yet claimed</x:v>
+        <x:v>Draft path closed; Spurs season bridge remains</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9524,7 +10729,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -9554,171 +10759,297 @@
       </x:c>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="56" t="str">
+      <x:c r="A5" s="51" t="str">
         <x:v>S01</x:v>
       </x:c>
-      <x:c r="B5" s="56" t="str">
+      <x:c r="B5" s="51" t="str">
         <x:v>NBA Stats — Atlanta schedule</x:v>
       </x:c>
-      <x:c r="C5" s="56" t="str">
+      <x:c r="C5" s="51" t="str">
         <x:v>82-game official schedule baseline</x:v>
       </x:c>
-      <x:c r="D5" s="56" t="str">
+      <x:c r="D5" s="51" t="str">
         <x:v>https://www.nba.com/stats/team/1610612737/schedule?Season=2018-19</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="56" t="str">
+      <x:c r="A6" s="51" t="str">
         <x:v>S02</x:v>
       </x:c>
-      <x:c r="B6" s="56" t="str">
+      <x:c r="B6" s="51" t="str">
         <x:v>ESPN — Atlanta schedule</x:v>
       </x:c>
-      <x:c r="C6" s="56" t="str">
+      <x:c r="C6" s="51" t="str">
         <x:v>Scores/order cross-check; timezone dates not authoritative</x:v>
       </x:c>
-      <x:c r="D6" s="56" t="str">
+      <x:c r="D6" s="51" t="str">
         <x:v>https://www.espn.com/nba/team/schedule?name=ATL&amp;season=2019&amp;seasontype=2</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
-      <x:c r="A7" s="56" t="str">
+      <x:c r="A7" s="51" t="str">
         <x:v>S03</x:v>
       </x:c>
-      <x:c r="B7" s="56" t="str">
+      <x:c r="B7" s="51" t="str">
         <x:v>Basketball-Reference — Atlanta schedule</x:v>
       </x:c>
-      <x:c r="C7" s="56" t="str">
+      <x:c r="C7" s="51" t="str">
         <x:v>29-53 and game-log cross-check</x:v>
       </x:c>
-      <x:c r="D7" s="56" t="str">
+      <x:c r="D7" s="51" t="str">
         <x:v>https://www.basketball-reference.com/teams/ATL/2019_games.html</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
-      <x:c r="A8" s="56" t="str">
+      <x:c r="A8" s="51" t="str">
         <x:v>S04</x:v>
       </x:c>
-      <x:c r="B8" s="56" t="str">
+      <x:c r="B8" s="51" t="str">
         <x:v>NBA Stats — Atlanta player totals</x:v>
       </x:c>
-      <x:c r="C8" s="56" t="str">
+      <x:c r="C8" s="51" t="str">
         <x:v>Roster GP/GS/minutes baseline</x:v>
       </x:c>
-      <x:c r="D8" s="56" t="str">
+      <x:c r="D8" s="51" t="str">
         <x:v>https://www.nba.com/stats/players/traditional?Season=2018-19&amp;SeasonType=Regular%20Season&amp;TeamID=1610612737&amp;PerMode=Totals</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="56" t="str">
+      <x:c r="A9" s="51" t="str">
         <x:v>S05</x:v>
       </x:c>
-      <x:c r="B9" s="56" t="str">
+      <x:c r="B9" s="51" t="str">
         <x:v>Hawks — Spellman injury update</x:v>
       </x:c>
-      <x:c r="C9" s="56" t="str">
+      <x:c r="C9" s="51" t="str">
         <x:v>March 1 high ankle sprain; not copied to protagonist</x:v>
       </x:c>
-      <x:c r="D9" s="56" t="str">
+      <x:c r="D9" s="51" t="str">
         <x:v>https://www.nba.com/hawks/news/omari-spellman-injury-update</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="56" t="str">
+      <x:c r="A10" s="51" t="str">
         <x:v>S06</x:v>
       </x:c>
-      <x:c r="B10" s="56" t="str">
+      <x:c r="B10" s="51" t="str">
         <x:v>NBA G League — Spellman</x:v>
       </x:c>
-      <x:c r="C10" s="56" t="str">
+      <x:c r="C10" s="51" t="str">
         <x:v>2018-19: 3 starts, 32.7 MPG</x:v>
       </x:c>
-      <x:c r="D10" s="56" t="str">
+      <x:c r="D10" s="51" t="str">
         <x:v>https://gleague.nba.com/player/1629016</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="56" t="str">
+      <x:c r="A11" s="51" t="str">
         <x:v>S07</x:v>
       </x:c>
-      <x:c r="B11" s="56" t="str">
+      <x:c r="B11" s="51" t="str">
         <x:v>Hawks — 2019 lottery odds explained</x:v>
       </x:c>
-      <x:c r="C11" s="56" t="str">
+      <x:c r="C11" s="51" t="str">
         <x:v>Atlanta/Dallas pick protection and odds baseline</x:v>
       </x:c>
-      <x:c r="D11" s="56" t="str">
+      <x:c r="D11" s="51" t="str">
         <x:v>https://www.nba.com/hawks/features/hawks-lottery-odds-explained</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="56" t="str">
+      <x:c r="A12" s="51" t="str">
         <x:v>S08</x:v>
       </x:c>
-      <x:c r="B12" s="56" t="str">
+      <x:c r="B12" s="51" t="str">
         <x:v>NBA Communications — 2019 tiebreakers</x:v>
       </x:c>
-      <x:c r="C12" s="56" t="str">
+      <x:c r="C12" s="51" t="str">
         <x:v>Lottery teams, inverse order, tied combinations</x:v>
       </x:c>
-      <x:c r="D12" s="56" t="str">
+      <x:c r="D12" s="51" t="str">
         <x:v>https://pr.nba.com/2019-nba-draft-tiebreakers/</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="56" t="str">
+      <x:c r="A13" s="51" t="str">
         <x:v>S09</x:v>
       </x:c>
-      <x:c r="B13" s="56" t="str">
+      <x:c r="B13" s="51" t="str">
         <x:v>NBA — 2019 lottery result</x:v>
       </x:c>
-      <x:c r="C13" s="56" t="str">
+      <x:c r="C13" s="51" t="str">
         <x:v>Actual draw baseline only</x:v>
       </x:c>
-      <x:c r="D13" s="56" t="str">
+      <x:c r="D13" s="51" t="str">
         <x:v>https://www.nba.com/news/pelicans-win-nba-draft-lottery</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="56" t="str">
+      <x:c r="A14" s="51" t="str">
         <x:v>S10</x:v>
       </x:c>
-      <x:c r="B14" s="56" t="str">
+      <x:c r="B14" s="51" t="str">
         <x:v>Hawks — Oct. 24 Dallas game</x:v>
       </x:c>
-      <x:c r="C14" s="56" t="str">
+      <x:c r="C14" s="51" t="str">
         <x:v>Atlanta 111-104 Dallas official game page</x:v>
       </x:c>
-      <x:c r="D14" s="56" t="str">
+      <x:c r="D14" s="51" t="str">
         <x:v>https://www.nba.com/hawks/game/0021800052-mavericks-vs-hawks-atlanta-ga-10-24-2018</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="56" t="str">
+      <x:c r="A15" s="51" t="str">
         <x:v>S11</x:v>
       </x:c>
-      <x:c r="B15" s="56" t="str">
+      <x:c r="B15" s="51" t="str">
         <x:v>Mavericks — Dec. 12 Atlanta game</x:v>
       </x:c>
-      <x:c r="C15" s="56" t="str">
+      <x:c r="C15" s="51" t="str">
         <x:v>Dallas 114-107 Atlanta official recap</x:v>
       </x:c>
-      <x:c r="D15" s="56" t="str">
+      <x:c r="D15" s="51" t="str">
         <x:v>https://www.nba.com/mavs/mavs-get-a-spark-from-carlisle-and-rallied-for-a-114-107-victory-over-the-hawks</x:v>
       </x:c>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="56" t="str">
+      <x:c r="A16" s="51" t="str">
         <x:v>S12</x:v>
       </x:c>
-      <x:c r="B16" s="56" t="str">
+      <x:c r="B16" s="51" t="str">
         <x:v>NBA — 2018 Atlanta draft</x:v>
       </x:c>
-      <x:c r="C16" s="56" t="str">
+      <x:c r="C16" s="51" t="str">
         <x:v>Actual 30th pick was Spellman</x:v>
       </x:c>
-      <x:c r="D16" s="56" t="str">
+      <x:c r="D16" s="51" t="str">
         <x:v>https://www.nba.com/hawks/news/hawks-acquire-trae-young-select-kevin-huerter-omari-spellman-2018-nba-draft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="51" t="str">
+        <x:v>S13</x:v>
+      </x:c>
+      <x:c r="B17" s="51" t="str">
+        <x:v>NBA — 2018 Draft Trade Tracker</x:v>
+      </x:c>
+      <x:c r="C17" s="51" t="str">
+        <x:v>Actual picks, rights trades, and destination teams</x:v>
+      </x:c>
+      <x:c r="D17" s="51" t="str">
+        <x:v>https://www.nba.com/2018-draft-trade-tracker</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="51" t="str">
+        <x:v>S14</x:v>
+      </x:c>
+      <x:c r="B18" s="51" t="str">
+        <x:v>San Antonio Express-News — Spurs workout target</x:v>
+      </x:c>
+      <x:c r="C18" s="51" t="str">
+        <x:v>Spellman worked out for Spurs; second workout interest</x:v>
+      </x:c>
+      <x:c r="D18" s="51" t="str">
+        <x:v>https://www.expressnews.com/spurs-nation/article/Spurs-target-Villanova-s-Spellman-others-for-12994749.php</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="51" t="str">
+        <x:v>S15</x:v>
+      </x:c>
+      <x:c r="B19" s="51" t="str">
+        <x:v>Sports Illustrated — final 2018 mock</x:v>
+      </x:c>
+      <x:c r="C19" s="51" t="str">
+        <x:v>Spellman #44 range; Spurs fit; Metu second-round range</x:v>
+      </x:c>
+      <x:c r="D19" s="51" t="str">
+        <x:v>https://www.si.com/nba/2018/06/21/nba-mock-draft-2018-trade-rumors-final-picks-deandre-ayton-trae-young</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="51" t="str">
+        <x:v>S16</x:v>
+      </x:c>
+      <x:c r="B20" s="51" t="str">
+        <x:v>Wizards — Issuf Sanon plan</x:v>
+      </x:c>
+      <x:c r="C20" s="51" t="str">
+        <x:v>Washington explicitly preferred an overseas stash</x:v>
+      </x:c>
+      <x:c r="D20" s="51" t="str">
+        <x:v>https://www.nba.com/wizards/wizards-plan-second-round-pick-issuf-sanon</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="51" t="str">
+        <x:v>S17</x:v>
+      </x:c>
+      <x:c r="B21" s="51" t="str">
+        <x:v>Nets — Rodions Kurucs scouting history</x:v>
+      </x:c>
+      <x:c r="C21" s="51" t="str">
+        <x:v>Brooklyn's long-running Kurucs evaluation</x:v>
+      </x:c>
+      <x:c r="D21" s="51" t="str">
+        <x:v>https://www.nba.com/nets/news/feature/2018/12/28/brooklyn-nets-rookie-rodions-kurucs-had-a-breakout-month-in-december</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="51" t="str">
+        <x:v>S18</x:v>
+      </x:c>
+      <x:c r="B22" s="51" t="str">
+        <x:v>NBA — 2018 big-board tiers</x:v>
+      </x:c>
+      <x:c r="C22" s="51" t="str">
+        <x:v>Spalding in drafted second-round tier; Welsh in the mix</x:v>
+      </x:c>
+      <x:c r="D22" s="51" t="str">
+        <x:v>https://www.nba.com/da-big-board-bigs-2018-draft</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="51" t="str">
+        <x:v>S19</x:v>
+      </x:c>
+      <x:c r="B23" s="51" t="str">
+        <x:v>Nuggets — Thomas Welsh two-way</x:v>
+      </x:c>
+      <x:c r="C23" s="51" t="str">
+        <x:v>Actual Welsh two-way destination used as role-preservation baseline</x:v>
+      </x:c>
+      <x:c r="D23" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/thomas-welsh-signs-two-way-contract-071918</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="51" t="str">
+        <x:v>S20</x:v>
+      </x:c>
+      <x:c r="B24" s="51" t="str">
+        <x:v>Basketball-Reference — Chimezie Metu</x:v>
+      </x:c>
+      <x:c r="C24" s="51" t="str">
+        <x:v>2018-19 San Antonio: 29 games, 5.0 MPG (145 minutes)</x:v>
+      </x:c>
+      <x:c r="D24" s="51" t="str">
+        <x:v>https://www.basketball-reference.com/players/m/metuch01.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="51" t="str">
+        <x:v>S21</x:v>
+      </x:c>
+      <x:c r="B25" s="51" t="str">
+        <x:v>Pounding the Rock — Metu season review</x:v>
+      </x:c>
+      <x:c r="C25" s="51" t="str">
+        <x:v>Most rookie NBA minutes came in garbage time; Austin was primary development venue</x:v>
+      </x:c>
+      <x:c r="D25" s="51" t="str">
+        <x:v>https://www.poundingtherock.com/2019/5/4/18523491/2018-2019-spurs-player-reviews-chimezie-metu</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9727,7 +11058,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re135e721277e4331"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa46802df9134e72"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Lock Spurs second-team impact baseline
</commit_message>
<xml_diff>
--- a/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
+++ b/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
@@ -2,13 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R243ec70f0c2544d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="R004ae6c0cc164082"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="R89934bb09586473b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R4a11c7dc755f4e8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="5" r:id="Rdfaeae280acc4ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="6" r:id="Ra5b8f023a20e46c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="7" r:id="R41ecceb893434cf6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R366e1f9bc1784d4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="Rac03984f160d43c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="Ra5b04d9f3a924551"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R3e5d45d21e1545b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurs Impact" sheetId="5" r:id="R60f9cfc284d9453b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="6" r:id="Ra11d836a74e4428d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="7" r:id="Rc70dc5e77334451b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R342fc8719a2a4474"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -25,7 +26,7 @@
     <x:numFmt numFmtId="202" formatCode="0.0"/>
     <x:numFmt numFmtId="203" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -84,6 +85,12 @@
     </x:font>
     <x:font>
       <x:sz val="9"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF17223B"/>
       <x:name val="Aptos"/>
     </x:font>
     <x:font>
@@ -175,7 +182,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="60">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -288,12 +295,27 @@
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <x:xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -399,7 +421,23 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SourceTable" displayName="SourceTable" ref="A4:D25" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="SpursAssignmentTable" displayName="SpursAssignmentTable" ref="A15:H34" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
+    <x:tableColumn id="1" name="Window"/>
+    <x:tableColumn id="2" name="Assign date"/>
+    <x:tableColumn id="3" name="Recall date"/>
+    <x:tableColumn id="4" name="Calendar days"/>
+    <x:tableColumn id="5" name="Entry"/>
+    <x:tableColumn id="6" name="Exit"/>
+    <x:tableColumn id="7" name="Contract/status"/>
+    <x:tableColumn id="8" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourceTable" displayName="SourceTable" ref="A4:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Source"/>
@@ -617,7 +655,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="18" t="str">
-        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.2</x:v>
+        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.3</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -652,7 +690,7 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>BASELINE_PASS / SECOND_TEAM_IMPACT_HOLD</x:v>
+        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
         <x:v>Canon</x:v>
@@ -952,7 +990,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Spellman's destination is resolved at San Antonio #49. The 2019 standings/lottery cannot be FINAL until the Spurs' 2018-19 impact is closed.</x:v>
+        <x:v>Spellman's San Antonio #49 baseline role is closed at Metu's low-leverage slot. Any minutes above 145.4 need a dated donor; competitive stints trigger outcome review.</x:v>
       </x:c>
       <x:c r="C18" s="22"/>
       <x:c r="D18" s="22"/>
@@ -8024,7 +8062,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R187056fa3cab45d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70e1b02e502342a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9063,7 +9101,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5d4fefc5fb924228"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0edad3bb7357419f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9116,7 +9154,7 @@
         <x:v>Next blocker</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>Spurs 2018-19 impact</x:v>
+        <x:v>Dallas/Denver contracts</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -9848,10 +9886,10 @@
         <x:v>Spellman worked out for San Antonio and fit its spacing/IQ profile.</x:v>
       </x:c>
       <x:c r="J26" s="53" t="str">
-        <x:v>Spurs 2018-19 impact HOLD</x:v>
+        <x:v>Spurs baseline role PASS; outcomes HOLD</x:v>
       </x:c>
       <x:c r="K26" s="53" t="str">
-        <x:v>S14/S15</x:v>
+        <x:v>S14/S15/S22</x:v>
       </x:c>
     </x:row>
     <x:row r="27">
@@ -10245,12 +10283,1017 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd845085108c84979"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb23b2dbd43ef4286"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="27" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="27" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="24" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>SAN ANTONIO 2018-19 — SECOND-TEAM IMPACT FIREWALL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="56" t="str">
+        <x:v>Actual Spurs</x:v>
+      </x:c>
+      <x:c r="B4" s="56" t="str">
+        <x:v>48-34</x:v>
+      </x:c>
+      <x:c r="C4" s="56" t="str">
+        <x:v>Metu NBA</x:v>
+      </x:c>
+      <x:c r="D4" s="56" t="str">
+        <x:v>29 G / 145.4 MIN</x:v>
+      </x:c>
+      <x:c r="E4" s="56" t="str">
+        <x:v>Metu Austin</x:v>
+      </x:c>
+      <x:c r="F4" s="56" t="str">
+        <x:v>26 G / 710.4 MIN</x:v>
+      </x:c>
+      <x:c r="G4" s="56" t="str">
+        <x:v>CF base</x:v>
+      </x:c>
+      <x:c r="H4" s="56" t="str">
+        <x:v>29 G / 145.4 MIN</x:v>
+      </x:c>
+      <x:c r="I4" s="56" t="str">
+        <x:v>ATL series</x:v>
+      </x:c>
+      <x:c r="J4" s="56" t="str">
+        <x:v>2 G / 0 MIN</x:v>
+      </x:c>
+      <x:c r="K4" s="56" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="L4" s="56" t="str">
+        <x:v>BASELINE_ROLE_PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="57"/>
+      <x:c r="B5" s="57"/>
+      <x:c r="C5" s="57"/>
+      <x:c r="D5" s="57"/>
+      <x:c r="E5" s="57"/>
+      <x:c r="F5" s="57"/>
+      <x:c r="G5" s="57"/>
+      <x:c r="H5" s="57"/>
+      <x:c r="I5" s="57"/>
+      <x:c r="J5" s="57"/>
+      <x:c r="K5" s="57"/>
+      <x:c r="L5" s="57"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="40" t="str">
+        <x:v>Scenario</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>NBA GP</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>NBA MPG</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="str">
+        <x:v>NBA MIN</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="str">
+        <x:v>Starts</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="str">
+        <x:v>Austin GP</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="str">
+        <x:v>Result rule</x:v>
+      </x:c>
+      <x:c r="H6" s="40" t="str">
+        <x:v>Required evidence</x:v>
+      </x:c>
+      <x:c r="I6" s="57"/>
+      <x:c r="J6" s="57"/>
+      <x:c r="K6" s="57"/>
+      <x:c r="L6" s="57"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="58" t="str">
+        <x:v>LOW</x:v>
+      </x:c>
+      <x:c r="B7" s="58" t="n">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="C7" s="58" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="D7" s="58" t="n">
+        <x:v>120</x:v>
+      </x:c>
+      <x:c r="E7" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F7" s="58" t="n">
+        <x:v>28</x:v>
+      </x:c>
+      <x:c r="G7" s="58" t="str">
+        <x:v>No automatic game changes</x:v>
+      </x:c>
+      <x:c r="H7" s="58" t="str">
+        <x:v>Stay inside Metu/deep-reserve slot</x:v>
+      </x:c>
+      <x:c r="I7" s="57"/>
+      <x:c r="J7" s="57"/>
+      <x:c r="K7" s="57"/>
+      <x:c r="L7" s="57"/>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="58" t="str">
+        <x:v>BASE</x:v>
+      </x:c>
+      <x:c r="B8" s="58" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="C8" s="58" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="D8" s="58" t="n">
+        <x:v>145.4</x:v>
+      </x:c>
+      <x:c r="E8" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="58" t="n">
+        <x:v>26</x:v>
+      </x:c>
+      <x:c r="G8" s="58" t="str">
+        <x:v>No automatic game changes</x:v>
+      </x:c>
+      <x:c r="H8" s="58" t="str">
+        <x:v>Metu actual role baseline</x:v>
+      </x:c>
+      <x:c r="I8" s="57"/>
+      <x:c r="J8" s="57"/>
+      <x:c r="K8" s="57"/>
+      <x:c r="L8" s="57"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="58" t="str">
+        <x:v>HIGH</x:v>
+      </x:c>
+      <x:c r="B9" s="58" t="n">
+        <x:v>31</x:v>
+      </x:c>
+      <x:c r="C9" s="58" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="D9" s="58" t="n">
+        <x:v>180</x:v>
+      </x:c>
+      <x:c r="E9" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F9" s="58" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="G9" s="58" t="str">
+        <x:v>GAME_REVIEW if competitive</x:v>
+      </x:c>
+      <x:c r="H9" s="58" t="str">
+        <x:v>Dated donor required above 145.4</x:v>
+      </x:c>
+      <x:c r="I9" s="57"/>
+      <x:c r="J9" s="57"/>
+      <x:c r="K9" s="57"/>
+      <x:c r="L9" s="57"/>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="57"/>
+      <x:c r="B10" s="57"/>
+      <x:c r="C10" s="57"/>
+      <x:c r="D10" s="57"/>
+      <x:c r="E10" s="57"/>
+      <x:c r="F10" s="57"/>
+      <x:c r="G10" s="57"/>
+      <x:c r="H10" s="57"/>
+      <x:c r="I10" s="57"/>
+      <x:c r="J10" s="57"/>
+      <x:c r="K10" s="57"/>
+      <x:c r="L10" s="57"/>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="40" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="B11" s="40" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="C11" s="40" t="str">
+        <x:v>Opponent</x:v>
+      </x:c>
+      <x:c r="D11" s="40" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="E11" s="40" t="str">
+        <x:v>SAS Pts</x:v>
+      </x:c>
+      <x:c r="F11" s="40" t="str">
+        <x:v>ATL Pts</x:v>
+      </x:c>
+      <x:c r="G11" s="40" t="str">
+        <x:v>Margin</x:v>
+      </x:c>
+      <x:c r="H11" s="40" t="str">
+        <x:v>Metu roster</x:v>
+      </x:c>
+      <x:c r="I11" s="40" t="str">
+        <x:v>Metu status</x:v>
+      </x:c>
+      <x:c r="J11" s="40" t="str">
+        <x:v>Spurs-side CF contact</x:v>
+      </x:c>
+      <x:c r="K11" s="40" t="str">
+        <x:v>Outcome status</x:v>
+      </x:c>
+      <x:c r="L11" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="59" t="n">
+        <x:v>43530.5</x:v>
+      </x:c>
+      <x:c r="B12" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="C12" s="58" t="str">
+        <x:v>Atlanta Hawks</x:v>
+      </x:c>
+      <x:c r="D12" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E12" s="58" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="F12" s="58" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="G12" s="58" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H12" s="58" t="str">
+        <x:v>NBA roster</x:v>
+      </x:c>
+      <x:c r="I12" s="58" t="str">
+        <x:v>DNP-CD / 0</x:v>
+      </x:c>
+      <x:c r="J12" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K12" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L12" s="58" t="str">
+        <x:v>S25</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="59" t="n">
+        <x:v>43557.5</x:v>
+      </x:c>
+      <x:c r="B13" s="58" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="C13" s="58" t="str">
+        <x:v>Atlanta Hawks</x:v>
+      </x:c>
+      <x:c r="D13" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E13" s="58" t="n">
+        <x:v>117</x:v>
+      </x:c>
+      <x:c r="F13" s="58" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="G13" s="58" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="H13" s="58" t="str">
+        <x:v>NBA roster</x:v>
+      </x:c>
+      <x:c r="I13" s="58" t="str">
+        <x:v>Inactive/0</x:v>
+      </x:c>
+      <x:c r="J13" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K13" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L13" s="58" t="str">
+        <x:v>S26</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="57"/>
+      <x:c r="B14" s="57"/>
+      <x:c r="C14" s="57"/>
+      <x:c r="D14" s="57"/>
+      <x:c r="E14" s="57"/>
+      <x:c r="F14" s="57"/>
+      <x:c r="G14" s="57"/>
+      <x:c r="H14" s="57"/>
+      <x:c r="I14" s="57"/>
+      <x:c r="J14" s="57"/>
+      <x:c r="K14" s="57"/>
+      <x:c r="L14" s="57"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="40" t="str">
+        <x:v>Window</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>Assign date</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>Recall date</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>Calendar days</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>Entry</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>Exit</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>Contract/status</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+      <x:c r="I15" s="57"/>
+      <x:c r="J15" s="40" t="str">
+        <x:v>Audit</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="n">
+        <x:v>43398.5</x:v>
+      </x:c>
+      <x:c r="C16" s="59" t="n">
+        <x:v>43400.5</x:v>
+      </x:c>
+      <x:c r="D16" s="58" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E16" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F16" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G16" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H16" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I16" s="57"/>
+      <x:c r="J16" s="58" t="str">
+        <x:v>Assignment windows</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="n">
+        <x:f>COUNTA(A16:A34)</x:f>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:f>IF(K16=19,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="58" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="n">
+        <x:v>43409.5</x:v>
+      </x:c>
+      <x:c r="C17" s="59" t="n">
+        <x:v>43409.5</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E17" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F17" s="58" t="str">
+        <x:v>Same-day recall</x:v>
+      </x:c>
+      <x:c r="G17" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H17" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I17" s="57"/>
+      <x:c r="J17" s="58" t="str">
+        <x:v>Direct games</x:v>
+      </x:c>
+      <x:c r="K17" s="58" t="n">
+        <x:f>COUNTA(A12:A13)</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L17" s="58" t="str">
+        <x:f>IF(K17=2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="58" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="n">
+        <x:v>43412.5</x:v>
+      </x:c>
+      <x:c r="C18" s="59" t="n">
+        <x:v>43412.5</x:v>
+      </x:c>
+      <x:c r="D18" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E18" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F18" s="58" t="str">
+        <x:v>Same-day recall</x:v>
+      </x:c>
+      <x:c r="G18" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H18" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I18" s="57"/>
+      <x:c r="J18" s="58" t="str">
+        <x:v>Direct Metu minutes</x:v>
+      </x:c>
+      <x:c r="K18" s="58" t="n">
+        <x:f>0</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L18" s="58" t="str">
+        <x:f>IF(K18=0,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="58" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="B19" s="59" t="n">
+        <x:v>43424.5</x:v>
+      </x:c>
+      <x:c r="C19" s="59" t="n">
+        <x:v>43425.5</x:v>
+      </x:c>
+      <x:c r="D19" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E19" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F19" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G19" s="58" t="str">
+        <x:v>Second reported assignment</x:v>
+      </x:c>
+      <x:c r="H19" s="58" t="str">
+        <x:v>S22/S24</x:v>
+      </x:c>
+      <x:c r="I19" s="57"/>
+      <x:c r="J19" s="58" t="str">
+        <x:v>Base minutes</x:v>
+      </x:c>
+      <x:c r="K19" s="58" t="n">
+        <x:f>D8</x:f>
+        <x:v>145.4</x:v>
+      </x:c>
+      <x:c r="L19" s="58" t="str">
+        <x:f>IF(ABS(K19-145.4)&lt;0.01,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="58" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B20" s="59" t="n">
+        <x:v>43435.5</x:v>
+      </x:c>
+      <x:c r="C20" s="59" t="n">
+        <x:v>43436.5</x:v>
+      </x:c>
+      <x:c r="D20" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E20" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F20" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G20" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H20" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I20" s="57"/>
+      <x:c r="J20" s="58" t="str">
+        <x:v>High-base excess</x:v>
+      </x:c>
+      <x:c r="K20" s="58" t="n">
+        <x:f>D9-D8</x:f>
+        <x:v>34.599999999999994</x:v>
+      </x:c>
+      <x:c r="L20" s="58" t="str">
+        <x:f>IF(ABS(K20-34.6)&lt;0.01,"DONOR REQUIRED","CHECK")</x:f>
+        <x:v>DONOR REQUIRED</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="58" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="B21" s="59" t="n">
+        <x:v>43442.5</x:v>
+      </x:c>
+      <x:c r="C21" s="59" t="n">
+        <x:v>43443.5</x:v>
+      </x:c>
+      <x:c r="D21" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E21" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F21" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G21" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H21" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I21" s="57"/>
+      <x:c r="J21" s="58" t="str">
+        <x:v>Outcome lock</x:v>
+      </x:c>
+      <x:c r="K21" s="58" t="str">
+        <x:f>IF(K18=0,"SPURS-SIDE DIRECT PASS","REVIEW")</x:f>
+        <x:v>SPURS-SIDE DIRECT PASS</x:v>
+      </x:c>
+      <x:c r="L21" s="58" t="str">
+        <x:f>IF(K21="SPURS-SIDE DIRECT PASS","PASS","HOLD")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="58" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="B22" s="59" t="n">
+        <x:v>43448.5</x:v>
+      </x:c>
+      <x:c r="C22" s="59" t="n">
+        <x:v>43457.5</x:v>
+      </x:c>
+      <x:c r="D22" s="58" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E22" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F22" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G22" s="58" t="str">
+        <x:v>Development window</x:v>
+      </x:c>
+      <x:c r="H22" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I22" s="57"/>
+      <x:c r="J22" s="57"/>
+      <x:c r="K22" s="57"/>
+      <x:c r="L22" s="57"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="58" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="B23" s="59" t="n">
+        <x:v>43461.5</x:v>
+      </x:c>
+      <x:c r="C23" s="59" t="n">
+        <x:v>43468.5</x:v>
+      </x:c>
+      <x:c r="D23" s="58" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E23" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F23" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G23" s="58" t="str">
+        <x:v>Development window</x:v>
+      </x:c>
+      <x:c r="H23" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I23" s="57"/>
+      <x:c r="J23" s="60" t="str">
+        <x:v>48-34 remains BASELINE, not a locked counterfactual result. Atlanta-side player impact is still HOLD.</x:v>
+      </x:c>
+      <x:c r="K23" s="60"/>
+      <x:c r="L23" s="60"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="58" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="B24" s="59" t="n">
+        <x:v>43470.5</x:v>
+      </x:c>
+      <x:c r="C24" s="59" t="n">
+        <x:v>43470.5</x:v>
+      </x:c>
+      <x:c r="D24" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E24" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F24" s="58" t="str">
+        <x:v>Same-day recall</x:v>
+      </x:c>
+      <x:c r="G24" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H24" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I24" s="57"/>
+      <x:c r="J24" s="57"/>
+      <x:c r="K24" s="57"/>
+      <x:c r="L24" s="57"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="58" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="B25" s="59" t="n">
+        <x:v>43472.5</x:v>
+      </x:c>
+      <x:c r="C25" s="59" t="n">
+        <x:v>43482.5</x:v>
+      </x:c>
+      <x:c r="D25" s="58" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E25" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F25" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G25" s="58" t="str">
+        <x:v>Development window</x:v>
+      </x:c>
+      <x:c r="H25" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I25" s="57"/>
+      <x:c r="J25" s="57"/>
+      <x:c r="K25" s="57"/>
+      <x:c r="L25" s="57"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="58" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="B26" s="59" t="n">
+        <x:v>43484.5</x:v>
+      </x:c>
+      <x:c r="C26" s="59" t="n">
+        <x:v>43485.5</x:v>
+      </x:c>
+      <x:c r="D26" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E26" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F26" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G26" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H26" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I26" s="57"/>
+      <x:c r="J26" s="57"/>
+      <x:c r="K26" s="57"/>
+      <x:c r="L26" s="57"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="58" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="B27" s="59" t="n">
+        <x:v>43490.5</x:v>
+      </x:c>
+      <x:c r="C27" s="59" t="n">
+        <x:v>43491.5</x:v>
+      </x:c>
+      <x:c r="D27" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E27" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F27" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G27" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H27" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I27" s="57"/>
+      <x:c r="J27" s="57"/>
+      <x:c r="K27" s="57"/>
+      <x:c r="L27" s="57"/>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="58" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B28" s="59" t="n">
+        <x:v>43497.5</x:v>
+      </x:c>
+      <x:c r="C28" s="59" t="n">
+        <x:v>43498.5</x:v>
+      </x:c>
+      <x:c r="D28" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E28" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F28" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G28" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H28" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I28" s="57"/>
+      <x:c r="J28" s="57"/>
+      <x:c r="K28" s="57"/>
+      <x:c r="L28" s="57"/>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="58" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="B29" s="59" t="n">
+        <x:v>43506.5</x:v>
+      </x:c>
+      <x:c r="C29" s="59" t="n">
+        <x:v>43507.5</x:v>
+      </x:c>
+      <x:c r="D29" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E29" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F29" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G29" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H29" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I29" s="57"/>
+      <x:c r="J29" s="57"/>
+      <x:c r="K29" s="57"/>
+      <x:c r="L29" s="57"/>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="58" t="n">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B30" s="59" t="n">
+        <x:v>43524.5</x:v>
+      </x:c>
+      <x:c r="C30" s="59" t="n">
+        <x:v>43525.5</x:v>
+      </x:c>
+      <x:c r="D30" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E30" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F30" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G30" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H30" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I30" s="57"/>
+      <x:c r="J30" s="57"/>
+      <x:c r="K30" s="57"/>
+      <x:c r="L30" s="57"/>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="58" t="n">
+        <x:v>16</x:v>
+      </x:c>
+      <x:c r="B31" s="59" t="n">
+        <x:v>43531.5</x:v>
+      </x:c>
+      <x:c r="C31" s="59" t="n">
+        <x:v>43534.5</x:v>
+      </x:c>
+      <x:c r="D31" s="58" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E31" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F31" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G31" s="58" t="str">
+        <x:v>After Atlanta game</x:v>
+      </x:c>
+      <x:c r="H31" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I31" s="57"/>
+      <x:c r="J31" s="57"/>
+      <x:c r="K31" s="57"/>
+      <x:c r="L31" s="57"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="58" t="n">
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B32" s="59" t="n">
+        <x:v>43537.5</x:v>
+      </x:c>
+      <x:c r="C32" s="59" t="n">
+        <x:v>43539.5</x:v>
+      </x:c>
+      <x:c r="D32" s="58" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E32" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F32" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G32" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H32" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I32" s="57"/>
+      <x:c r="J32" s="57"/>
+      <x:c r="K32" s="57"/>
+      <x:c r="L32" s="57"/>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="58" t="n">
+        <x:v>18</x:v>
+      </x:c>
+      <x:c r="B33" s="59" t="n">
+        <x:v>43543.5</x:v>
+      </x:c>
+      <x:c r="C33" s="59" t="n">
+        <x:v>43544.5</x:v>
+      </x:c>
+      <x:c r="D33" s="58" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E33" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F33" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G33" s="58" t="str">
+        <x:v>NBA contract retained</x:v>
+      </x:c>
+      <x:c r="H33" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I33" s="57"/>
+      <x:c r="J33" s="57"/>
+      <x:c r="K33" s="57"/>
+      <x:c r="L33" s="57"/>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="58" t="n">
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B34" s="59" t="n">
+        <x:v>43545.5</x:v>
+      </x:c>
+      <x:c r="C34" s="59" t="n">
+        <x:v>43548.5</x:v>
+      </x:c>
+      <x:c r="D34" s="58" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E34" s="58" t="str">
+        <x:v>Austin assignment</x:v>
+      </x:c>
+      <x:c r="F34" s="58" t="str">
+        <x:v>Recall</x:v>
+      </x:c>
+      <x:c r="G34" s="58" t="str">
+        <x:v>Final logged window</x:v>
+      </x:c>
+      <x:c r="H34" s="58" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="I34" s="57"/>
+      <x:c r="J34" s="57"/>
+      <x:c r="K34" s="57"/>
+      <x:c r="L34" s="57"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:L2"/>
+    <x:mergeCell ref="J23:L23"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678b9e0485934009"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10316,10 +11359,10 @@
       <x:c r="D5" s="13" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="54" t="n">
+      <x:c r="E5" s="61" t="n">
         <x:v>0.105</x:v>
       </x:c>
-      <x:c r="F5" s="54" t="n">
+      <x:c r="F5" s="61" t="n">
         <x:v>0.4212</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
@@ -10348,10 +11391,10 @@
       <x:c r="D6" s="13" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E6" s="54" t="n">
+      <x:c r="E6" s="61" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="F6" s="54" t="n">
+      <x:c r="F6" s="61" t="n">
         <x:v>0.263</x:v>
       </x:c>
       <x:c r="G6" s="13" t="n">
@@ -10447,8 +11490,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="57" t="str">
-        <x:v>FINAL BLOCKER: Spellman is resolved to San Antonio #49; close the Spurs' 2018-19 rotation and game impact before standings/lottery.</x:v>
+      <x:c r="A14" s="64" t="str">
+        <x:v>FINAL BLOCKER: Spurs baseline role is closed. Execute Atlanta player-game impacts and review any Spellman competitive stints before standings/lottery.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10462,7 +11505,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -10504,19 +11547,19 @@
         <x:v>G0</x:v>
       </x:c>
       <x:c r="B5" s="51" t="str">
-        <x:v>Spellman destination + second-team impact</x:v>
+        <x:v>Spellman destination + second-team baseline</x:v>
       </x:c>
       <x:c r="C5" s="51" t="str">
-        <x:v>Spellman → Spurs #49; Spurs impact not executed</x:v>
+        <x:v>Spurs #49; base 29 G/145.4 min; ATL series 0 min</x:v>
       </x:c>
       <x:c r="D5" s="53" t="str">
-        <x:v>PARTIAL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="E5" s="51" t="str">
-        <x:v>FINAL standings/lottery</x:v>
+        <x:v>None</x:v>
       </x:c>
       <x:c r="F5" s="51" t="str">
-        <x:v>Model Spurs 2018-19</x:v>
+        <x:v>Preserve role cap and donor trigger</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10700,25 +11743,25 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="59"/>
-      <x:c r="B15" s="59"/>
-      <x:c r="C15" s="59"/>
-      <x:c r="D15" s="59"/>
-      <x:c r="E15" s="59"/>
-      <x:c r="F15" s="59"/>
+      <x:c r="A15" s="66"/>
+      <x:c r="B15" s="66"/>
+      <x:c r="C15" s="66"/>
+      <x:c r="D15" s="66"/>
+      <x:c r="E15" s="66"/>
+      <x:c r="F15" s="66"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="50" t="str">
         <x:v>OVERALL</x:v>
       </x:c>
       <x:c r="B16" s="50" t="str">
-        <x:v>BASELINE_PASS / SECOND_TEAM_IMPACT_HOLD</x:v>
+        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C16" s="50"/>
       <x:c r="D16" s="50"/>
       <x:c r="E16" s="50"/>
       <x:c r="F16" s="50" t="str">
-        <x:v>Draft path closed; Spurs season bridge remains</x:v>
+        <x:v>Atlanta player-game and competitive-stint outcomes remain</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10729,7 +11772,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -11052,13 +12095,97 @@
         <x:v>https://www.poundingtherock.com/2019/5/4/18523491/2018-2019-spurs-player-reviews-chimezie-metu</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="51" t="str">
+        <x:v>S22</x:v>
+      </x:c>
+      <x:c r="B26" s="51" t="str">
+        <x:v>RealGM — Chimezie Metu profile</x:v>
+      </x:c>
+      <x:c r="C26" s="51" t="str">
+        <x:v>2018-19 NBA totals, Austin totals, and assignment/recall transaction log</x:v>
+      </x:c>
+      <x:c r="D26" s="51" t="str">
+        <x:v>https://basketball.realgm.com/player/Chimezie-Metu/Summary/76976</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="51" t="str">
+        <x:v>S23</x:v>
+      </x:c>
+      <x:c r="B27" s="51" t="str">
+        <x:v>Spurs — Metu signing</x:v>
+      </x:c>
+      <x:c r="C27" s="51" t="str">
+        <x:v>Second-round pick signed to an NBA multi-year contract, not a two-way</x:v>
+      </x:c>
+      <x:c r="D27" s="51" t="str">
+        <x:v>https://www.nba.com/spurs/news/spurs-sign-2018-second-round-pick-chimezie-metu</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="51" t="str">
+        <x:v>S24</x:v>
+      </x:c>
+      <x:c r="B28" s="51" t="str">
+        <x:v>Fox San Antonio — Nov. 20 assignment</x:v>
+      </x:c>
+      <x:c r="C28" s="51" t="str">
+        <x:v>Contemporary report identifies Metu's second Austin assignment and NBA baseline</x:v>
+      </x:c>
+      <x:c r="D28" s="51" t="str">
+        <x:v>https://foxsanantonio.com/sports/max-sports/spurs-assign-rookie-metu-to-g-league</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="51" t="str">
+        <x:v>S25</x:v>
+      </x:c>
+      <x:c r="B29" s="51" t="str">
+        <x:v>ESPN — 2019-03-06 Spurs at Atlanta</x:v>
+      </x:c>
+      <x:c r="C29" s="51" t="str">
+        <x:v>Spurs 111-104; Metu DNP-Coach's Decision</x:v>
+      </x:c>
+      <x:c r="D29" s="51" t="str">
+        <x:v>https://www.espn.com/nba/boxscore/_/gameId/401071641</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="51" t="str">
+        <x:v>S26</x:v>
+      </x:c>
+      <x:c r="B30" s="51" t="str">
+        <x:v>NBA Hawks — 2019-04-02 Atlanta at Spurs</x:v>
+      </x:c>
+      <x:c r="C30" s="51" t="str">
+        <x:v>Spurs 117-111; Metu recorded no minutes</x:v>
+      </x:c>
+      <x:c r="D30" s="51" t="str">
+        <x:v>https://www.nba.com/hawks/game/0021801162-hawks-vs-spurs-san-antonio-tx-04-02-2019</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="51" t="str">
+        <x:v>S27</x:v>
+      </x:c>
+      <x:c r="B31" s="51" t="str">
+        <x:v>Spurs — 2019 Metu Austin recap</x:v>
+      </x:c>
+      <x:c r="C31" s="51" t="str">
+        <x:v>2018-19 Austin: 26 games, 14.0/7.4/2.3 in 27.3 MPG</x:v>
+      </x:c>
+      <x:c r="D31" s="51" t="str">
+        <x:v>https://www.nba.com/spurs/news/san-antonio-assigns-chimezie-metu-austin-spurs-8</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:D2"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Raa46802df9134e72"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c25f5cf78044f3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Close Dallas and Denver cascade contract layers
</commit_message>
<xml_diff>
--- a/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
+++ b/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R366e1f9bc1784d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="Rac03984f160d43c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="Ra5b04d9f3a924551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R3e5d45d21e1545b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurs Impact" sheetId="5" r:id="R60f9cfc284d9453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="6" r:id="Ra11d836a74e4428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="7" r:id="Rc70dc5e77334451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R342fc8719a2a4474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R68f787c966524bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="R0da9e4168273453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="R9235d60d1db24783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R66f8d0ab790c4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurs Impact" sheetId="5" r:id="R30ddbd1fb9b245ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cascade Impact" sheetId="6" r:id="Rc3254edf00a34c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="7" r:id="R880401c26dbd44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="8" r:id="Rc96c56130c3c4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R5bb35b2c8e9a47f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -309,6 +310,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -437,7 +441,48 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourceTable" displayName="SourceTable" ref="A4:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CascadeContractTable" displayName="CascadeContractTable" ref="A6:M12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Team"/>
+    <x:tableColumn id="2" name="World"/>
+    <x:tableColumn id="3" name="Player"/>
+    <x:tableColumn id="4" name="Pick"/>
+    <x:tableColumn id="5" name="Contract layer"/>
+    <x:tableColumn id="6" name="Development path"/>
+    <x:tableColumn id="7" name="NBA GP"/>
+    <x:tableColumn id="8" name="NBA MIN"/>
+    <x:tableColumn id="9" name="G League GP"/>
+    <x:tableColumn id="10" name="Transaction"/>
+    <x:tableColumn id="11" name="Role status"/>
+    <x:tableColumn id="12" name="Escalation trigger"/>
+    <x:tableColumn id="13" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CascadeDirectGameTable" displayName="CascadeDirectGameTable" ref="A15:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Team"/>
+    <x:tableColumn id="2" name="Date"/>
+    <x:tableColumn id="3" name="Site"/>
+    <x:tableColumn id="4" name="Actual"/>
+    <x:tableColumn id="5" name="Team pts"/>
+    <x:tableColumn id="6" name="ATL pts"/>
+    <x:tableColumn id="7" name="Margin"/>
+    <x:tableColumn id="8" name="Replaced player"/>
+    <x:tableColumn id="9" name="Replaced MIN"/>
+    <x:tableColumn id="10" name="CF contact"/>
+    <x:tableColumn id="11" name="Outcome status"/>
+    <x:tableColumn id="12" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourceTable" displayName="SourceTable" ref="A4:D43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Source"/>
@@ -655,7 +700,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="18" t="str">
-        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.3</x:v>
+        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.4</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -690,13 +735,13 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
+        <x:v>CASCADE_CONTRACT_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
         <x:v>Canon</x:v>
       </x:c>
       <x:c r="D4" s="20" t="str">
-        <x:v>PROVISIONAL</x:v>
+        <x:v>v0.22 PARTIAL</x:v>
       </x:c>
       <x:c r="E4" s="20" t="str">
         <x:v>Manuscript</x:v>
@@ -990,7 +1035,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Spellman's San Antonio #49 baseline role is closed at Metu's low-leverage slot. Any minutes above 145.4 need a dated donor; competitive stints trigger outcome review.</x:v>
+        <x:v>The San Antonio, Dallas, and Denver replacement contract layers are closed. Each CF rookie starts inside the displaced player's team-specific role, not his old-team minutes.</x:v>
       </x:c>
       <x:c r="C18" s="22"/>
       <x:c r="D18" s="22"/>
@@ -1004,7 +1049,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>No counterfactual scores or results have been generated. Manual flips and close-game cherry-picking are prohibited.</x:v>
+        <x:v>Welsh cannot duplicate Denver's occupied two-way slot. His undrafted free-agent destination remains HOLD; no counterfactual scores or results have been generated.</x:v>
       </x:c>
       <x:c r="C19" s="22"/>
       <x:c r="D19" s="22"/>
@@ -8062,7 +8107,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70e1b02e502342a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1e5b9d80d449ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9101,7 +9146,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0edad3bb7357419f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d537aa0b8ad4ad9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9154,7 +9199,7 @@
         <x:v>Next blocker</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>Dallas/Denver contracts</x:v>
+        <x:v>Atlanta donor vector</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10131,10 +10176,10 @@
         <x:v>Metu is the displaced #49 athletic big and remains above this slot.</x:v>
       </x:c>
       <x:c r="J33" s="53" t="str">
-        <x:v>Dallas role/minutes HOLD</x:v>
+        <x:v>Dallas contract layer PASS; outcomes HOLD</x:v>
       </x:c>
       <x:c r="K33" s="53" t="str">
-        <x:v>S13/S15</x:v>
+        <x:v>S13/S15/S28/S29/S30</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -10201,10 +10246,10 @@
         <x:v>Spalding was graded in the drafted second-round big tier.</x:v>
       </x:c>
       <x:c r="J35" s="53" t="str">
-        <x:v>Denver role/two-way HOLD</x:v>
+        <x:v>Denver contract layer PASS; Welsh market HOLD</x:v>
       </x:c>
       <x:c r="K35" s="53" t="str">
-        <x:v>S18</x:v>
+        <x:v>S18/S31/S32/S33/S34</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -10283,7 +10328,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb23b2dbd43ef4286"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6d353ac21e5413d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11288,12 +11333,777 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678b9e0485934009"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5c86b37a184f22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="46" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>DALLAS / DENVER 2018-19 — CASCADE CONTRACT FIREWALL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="56" t="str">
+        <x:v>Dallas base</x:v>
+      </x:c>
+      <x:c r="B4" s="56" t="str">
+        <x:v>1 G / 1 MIN</x:v>
+      </x:c>
+      <x:c r="C4" s="56"/>
+      <x:c r="D4" s="56" t="str">
+        <x:v>Texas</x:v>
+      </x:c>
+      <x:c r="E4" s="56" t="str">
+        <x:v>29 G / 30.1 MPG</x:v>
+      </x:c>
+      <x:c r="F4" s="56"/>
+      <x:c r="G4" s="56" t="str">
+        <x:v>Denver base</x:v>
+      </x:c>
+      <x:c r="H4" s="56" t="str">
+        <x:v>11 G / 36 MIN</x:v>
+      </x:c>
+      <x:c r="I4" s="56"/>
+      <x:c r="J4" s="56" t="str">
+        <x:v>ATL series</x:v>
+      </x:c>
+      <x:c r="K4" s="56" t="str">
+        <x:v>4 G / 0 MIN</x:v>
+      </x:c>
+      <x:c r="L4" s="56" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="M4" s="56" t="str">
+        <x:v>CONTRACT_LAYER_PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="57"/>
+      <x:c r="B5" s="57"/>
+      <x:c r="C5" s="57"/>
+      <x:c r="D5" s="57"/>
+      <x:c r="E5" s="57"/>
+      <x:c r="F5" s="57"/>
+      <x:c r="G5" s="57"/>
+      <x:c r="H5" s="57"/>
+      <x:c r="I5" s="57"/>
+      <x:c r="J5" s="57"/>
+      <x:c r="K5" s="57"/>
+      <x:c r="L5" s="57"/>
+      <x:c r="M5" s="57"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="40" t="str">
+        <x:v>Team</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>World</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>Player</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="str">
+        <x:v>Pick</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="str">
+        <x:v>Contract layer</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="str">
+        <x:v>Development path</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="str">
+        <x:v>NBA GP</x:v>
+      </x:c>
+      <x:c r="H6" s="40" t="str">
+        <x:v>NBA MIN</x:v>
+      </x:c>
+      <x:c r="I6" s="40" t="str">
+        <x:v>G League GP</x:v>
+      </x:c>
+      <x:c r="J6" s="40" t="str">
+        <x:v>Transaction</x:v>
+      </x:c>
+      <x:c r="K6" s="40" t="str">
+        <x:v>Role status</x:v>
+      </x:c>
+      <x:c r="L6" s="40" t="str">
+        <x:v>Escalation trigger</x:v>
+      </x:c>
+      <x:c r="M6" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="61" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B7" s="61" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="C7" s="61" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="D7" s="61" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="str">
+        <x:v>Standard NBA</x:v>
+      </x:c>
+      <x:c r="F7" s="61" t="str">
+        <x:v>Texas assignment</x:v>
+      </x:c>
+      <x:c r="G7" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I7" s="61" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J7" s="61" t="str">
+        <x:v>Waived 2019-01-31</x:v>
+      </x:c>
+      <x:c r="K7" s="61" t="str">
+        <x:v>ACTUAL_REPLACED</x:v>
+      </x:c>
+      <x:c r="L7" s="61" t="str">
+        <x:v>Reference only</x:v>
+      </x:c>
+      <x:c r="M7" s="61" t="str">
+        <x:v>S28/S29/S30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="61" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B8" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C8" s="61" t="str">
+        <x:v>Chimezie Metu</x:v>
+      </x:c>
+      <x:c r="D8" s="61" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E8" s="61" t="str">
+        <x:v>Standard NBA layer</x:v>
+      </x:c>
+      <x:c r="F8" s="61" t="str">
+        <x:v>Texas assignment baseline</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J8" s="61" t="str">
+        <x:v>Jan. 31 waiver choice HOLD</x:v>
+      </x:c>
+      <x:c r="K8" s="61" t="str">
+        <x:v>CF_CHANGED_STANDARD</x:v>
+      </x:c>
+      <x:c r="L8" s="61" t="str">
+        <x:v>&gt;1 NBA MIN or a different waiver opens Dallas player-game review</x:v>
+      </x:c>
+      <x:c r="M8" s="61" t="str">
+        <x:v>S28/S29/S30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B9" s="61" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="C9" s="61" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="D9" s="61" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>Two-way</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>Capital City / Iowa</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J9" s="61" t="str">
+        <x:v>Two-way ended 2019-07-30</x:v>
+      </x:c>
+      <x:c r="K9" s="61" t="str">
+        <x:v>ACTUAL_REPLACED</x:v>
+      </x:c>
+      <x:c r="L9" s="61" t="str">
+        <x:v>Reference only</x:v>
+      </x:c>
+      <x:c r="M9" s="61" t="str">
+        <x:v>S31/S34/S35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B10" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C10" s="61" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="D10" s="61" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>Two-way (Welsh slot)</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>External G League assignment class</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J10" s="61" t="str">
+        <x:v>Season role baseline</x:v>
+      </x:c>
+      <x:c r="K10" s="61" t="str">
+        <x:v>CF_CHANGED_TWO_WAY</x:v>
+      </x:c>
+      <x:c r="L10" s="61" t="str">
+        <x:v>&gt;36 NBA MIN or different dates opens Denver player-game review</x:v>
+      </x:c>
+      <x:c r="M10" s="61" t="str">
+        <x:v>S31/S32/S33/S34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B11" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C11" s="61" t="str">
+        <x:v>DeVaughn Akoon-Purcell</x:v>
+      </x:c>
+      <x:c r="D11" s="61"/>
+      <x:c r="E11" s="61" t="str">
+        <x:v>Two-way</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>G League development</x:v>
+      </x:c>
+      <x:c r="G11" s="61"/>
+      <x:c r="H11" s="61"/>
+      <x:c r="I11" s="61"/>
+      <x:c r="J11" s="61" t="str">
+        <x:v>Actual second slot preserved</x:v>
+      </x:c>
+      <x:c r="K11" s="61" t="str">
+        <x:v>CF_PROTECTED_TWO_WAY</x:v>
+      </x:c>
+      <x:c r="L11" s="61" t="str">
+        <x:v>Do not displace without a new transaction cause</x:v>
+      </x:c>
+      <x:c r="M11" s="61" t="str">
+        <x:v>S32/S33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B12" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C12" s="61" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="D12" s="61"/>
+      <x:c r="E12" s="61" t="str">
+        <x:v>No Denver slot</x:v>
+      </x:c>
+      <x:c r="F12" s="61" t="str">
+        <x:v>Undrafted free-agent market</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="61" t="str">
+        <x:v>Destination unresolved</x:v>
+      </x:c>
+      <x:c r="K12" s="61" t="str">
+        <x:v>CF_OUT_NO_SLOT</x:v>
+      </x:c>
+      <x:c r="L12" s="61" t="str">
+        <x:v>Any NBA signing creates a new team-impact branch</x:v>
+      </x:c>
+      <x:c r="M12" s="61" t="str">
+        <x:v>S31/S32/S33/S35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="57"/>
+      <x:c r="B13" s="57"/>
+      <x:c r="C13" s="57"/>
+      <x:c r="D13" s="57"/>
+      <x:c r="E13" s="57"/>
+      <x:c r="F13" s="57"/>
+      <x:c r="G13" s="57"/>
+      <x:c r="H13" s="57"/>
+      <x:c r="I13" s="57"/>
+      <x:c r="J13" s="57"/>
+      <x:c r="K13" s="57"/>
+      <x:c r="L13" s="57"/>
+      <x:c r="M13" s="57"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="57"/>
+      <x:c r="B14" s="57"/>
+      <x:c r="C14" s="57"/>
+      <x:c r="D14" s="57"/>
+      <x:c r="E14" s="57"/>
+      <x:c r="F14" s="57"/>
+      <x:c r="G14" s="57"/>
+      <x:c r="H14" s="57"/>
+      <x:c r="I14" s="57"/>
+      <x:c r="J14" s="57"/>
+      <x:c r="K14" s="57"/>
+      <x:c r="L14" s="57"/>
+      <x:c r="M14" s="57"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="40" t="str">
+        <x:v>Team</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>Team pts</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>ATL pts</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>Margin</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>Replaced player</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>Replaced MIN</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>CF contact</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>Outcome status</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+      <x:c r="M15" s="57"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="58" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="n">
+        <x:v>43397.5</x:v>
+      </x:c>
+      <x:c r="C16" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D16" s="58" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E16" s="58" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="F16" s="58" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="G16" s="58" t="n">
+        <x:v>-7</x:v>
+      </x:c>
+      <x:c r="H16" s="58" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="I16" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>S10/S29</x:v>
+      </x:c>
+      <x:c r="M16" s="57"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="58" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="n">
+        <x:v>43446.5</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E17" s="58" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="F17" s="58" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="G17" s="58" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H17" s="58" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="I17" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K17" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L17" s="58" t="str">
+        <x:v>S11/S29</x:v>
+      </x:c>
+      <x:c r="M17" s="57"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="58" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="n">
+        <x:v>43419.5</x:v>
+      </x:c>
+      <x:c r="C18" s="58" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D18" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E18" s="58" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="F18" s="58" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="G18" s="58" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="H18" s="58" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="I18" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K18" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L18" s="58" t="str">
+        <x:v>S36/S37</x:v>
+      </x:c>
+      <x:c r="M18" s="57"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="58" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B19" s="59" t="n">
+        <x:v>43442.5</x:v>
+      </x:c>
+      <x:c r="C19" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D19" s="58" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E19" s="58" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F19" s="58" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G19" s="58" t="n">
+        <x:v>-8</x:v>
+      </x:c>
+      <x:c r="H19" s="58" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="I19" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K19" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L19" s="58" t="str">
+        <x:v>S38/S39</x:v>
+      </x:c>
+      <x:c r="M19" s="57"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="57"/>
+      <x:c r="B20" s="57"/>
+      <x:c r="C20" s="57"/>
+      <x:c r="D20" s="57"/>
+      <x:c r="E20" s="57"/>
+      <x:c r="F20" s="57"/>
+      <x:c r="G20" s="57"/>
+      <x:c r="H20" s="57"/>
+      <x:c r="I20" s="57"/>
+      <x:c r="J20" s="57"/>
+      <x:c r="K20" s="57"/>
+      <x:c r="L20" s="57"/>
+      <x:c r="M20" s="57"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="60" t="str">
+        <x:v>Dallas: Metu begins inside Spalding's standard-contract / Texas assignment slot; a different Jan. 31 waiver choice remains HOLD. Denver: Spalding takes Welsh's two-way slot, Akoon-Purcell keeps the other, and Welsh moves to the undrafted free-agent market. Any minutes above the displaced-player base reopen player-game review.</x:v>
+      </x:c>
+      <x:c r="B21" s="60"/>
+      <x:c r="C21" s="60"/>
+      <x:c r="D21" s="60"/>
+      <x:c r="E21" s="60"/>
+      <x:c r="F21" s="60"/>
+      <x:c r="G21" s="60"/>
+      <x:c r="H21" s="60"/>
+      <x:c r="I21" s="57"/>
+      <x:c r="J21" s="40" t="str">
+        <x:v>Audit</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="L21" s="40" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="M21" s="57"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="60"/>
+      <x:c r="B22" s="60"/>
+      <x:c r="C22" s="60"/>
+      <x:c r="D22" s="60"/>
+      <x:c r="E22" s="60"/>
+      <x:c r="F22" s="60"/>
+      <x:c r="G22" s="60"/>
+      <x:c r="H22" s="60"/>
+      <x:c r="I22" s="57"/>
+      <x:c r="J22" s="58" t="str">
+        <x:v>Changed contract chains</x:v>
+      </x:c>
+      <x:c r="K22" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_CHANGED_STANDARD")+COUNTIF(K7:K12,"CF_CHANGED_TWO_WAY")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L22" s="58" t="str">
+        <x:f>IF(K22=2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M22" s="57"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="60"/>
+      <x:c r="B23" s="60"/>
+      <x:c r="C23" s="60"/>
+      <x:c r="D23" s="60"/>
+      <x:c r="E23" s="60"/>
+      <x:c r="F23" s="60"/>
+      <x:c r="G23" s="60"/>
+      <x:c r="H23" s="60"/>
+      <x:c r="I23" s="57"/>
+      <x:c r="J23" s="58" t="str">
+        <x:v>Direct games</x:v>
+      </x:c>
+      <x:c r="K23" s="58" t="n">
+        <x:f>COUNTA(A16:A19)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L23" s="58" t="str">
+        <x:f>IF(K23=4,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M23" s="57"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="57"/>
+      <x:c r="B24" s="57"/>
+      <x:c r="C24" s="57"/>
+      <x:c r="D24" s="57"/>
+      <x:c r="E24" s="57"/>
+      <x:c r="F24" s="57"/>
+      <x:c r="G24" s="57"/>
+      <x:c r="H24" s="57"/>
+      <x:c r="I24" s="57"/>
+      <x:c r="J24" s="58" t="str">
+        <x:v>Direct replaced minutes</x:v>
+      </x:c>
+      <x:c r="K24" s="58" t="n">
+        <x:f>SUM(I16:I19)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="58" t="str">
+        <x:f>IF(K24=0,"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M24" s="57"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="57"/>
+      <x:c r="B25" s="57"/>
+      <x:c r="C25" s="57"/>
+      <x:c r="D25" s="57"/>
+      <x:c r="E25" s="57"/>
+      <x:c r="F25" s="57"/>
+      <x:c r="G25" s="57"/>
+      <x:c r="H25" s="57"/>
+      <x:c r="I25" s="57"/>
+      <x:c r="J25" s="58" t="str">
+        <x:v>Denver CF two-way slots</x:v>
+      </x:c>
+      <x:c r="K25" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_CHANGED_TWO_WAY")+COUNTIF(K7:K12,"CF_PROTECTED_TWO_WAY")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L25" s="58" t="str">
+        <x:f>IF(K25=2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M25" s="57"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="57"/>
+      <x:c r="B26" s="57"/>
+      <x:c r="C26" s="57"/>
+      <x:c r="D26" s="57"/>
+      <x:c r="E26" s="57"/>
+      <x:c r="F26" s="57"/>
+      <x:c r="G26" s="57"/>
+      <x:c r="H26" s="57"/>
+      <x:c r="I26" s="57"/>
+      <x:c r="J26" s="58" t="str">
+        <x:v>Welsh duplicate blocked</x:v>
+      </x:c>
+      <x:c r="K26" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_OUT_NO_SLOT")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L26" s="58" t="str">
+        <x:f>IF(K26=1,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M26" s="57"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="57"/>
+      <x:c r="B27" s="57"/>
+      <x:c r="C27" s="57"/>
+      <x:c r="D27" s="57"/>
+      <x:c r="E27" s="57"/>
+      <x:c r="F27" s="57"/>
+      <x:c r="G27" s="57"/>
+      <x:c r="H27" s="57"/>
+      <x:c r="I27" s="57"/>
+      <x:c r="J27" s="58" t="str">
+        <x:v>Outcome lock</x:v>
+      </x:c>
+      <x:c r="K27" s="58" t="str">
+        <x:f>IF(AND(K24=0,K25=2,K26=1),"CASCADE DIRECT PASS","REVIEW")</x:f>
+        <x:v>CASCADE DIRECT PASS</x:v>
+      </x:c>
+      <x:c r="L27" s="58" t="str">
+        <x:f>IF(K27="CASCADE DIRECT PASS","PASS","HOLD")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M27" s="57"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M2"/>
+    <x:mergeCell ref="A21:H23"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf6d880b3174b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3711a7d9ae4c67"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -11359,10 +12169,10 @@
       <x:c r="D5" s="13" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="n">
+      <x:c r="E5" s="62" t="n">
         <x:v>0.105</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="n">
+      <x:c r="F5" s="62" t="n">
         <x:v>0.4212</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
@@ -11391,10 +12201,10 @@
       <x:c r="D6" s="13" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E6" s="61" t="n">
+      <x:c r="E6" s="62" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="F6" s="61" t="n">
+      <x:c r="F6" s="62" t="n">
         <x:v>0.263</x:v>
       </x:c>
       <x:c r="G6" s="13" t="n">
@@ -11490,8 +12300,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="64" t="str">
-        <x:v>FINAL BLOCKER: Spurs baseline role is closed. Execute Atlanta player-game impacts and review any Spellman competitive stints before standings/lottery.</x:v>
+      <x:c r="A14" s="65" t="str">
+        <x:v>FINAL BLOCKER: Spurs, Dallas, and Denver contract layers are closed. Execute Atlanta player-game impacts and review only minutes beyond each displaced-player base before standings/lottery.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11505,7 +12315,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -11547,10 +12357,10 @@
         <x:v>G0</x:v>
       </x:c>
       <x:c r="B5" s="51" t="str">
-        <x:v>Spellman destination + second-team baseline</x:v>
+        <x:v>Changed-pick contract and direct-game baselines</x:v>
       </x:c>
       <x:c r="C5" s="51" t="str">
-        <x:v>Spurs #49; base 29 G/145.4 min; ATL series 0 min</x:v>
+        <x:v>Spurs 145.4 min; Dallas 1 min; Denver 36 min; ATL series all 0</x:v>
       </x:c>
       <x:c r="D5" s="53" t="str">
         <x:v>PASS</x:v>
@@ -11559,7 +12369,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="F5" s="51" t="str">
-        <x:v>Preserve role cap and donor trigger</x:v>
+        <x:v>Preserve team-specific caps and triggers</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11743,25 +12553,25 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="66"/>
-      <x:c r="B15" s="66"/>
-      <x:c r="C15" s="66"/>
-      <x:c r="D15" s="66"/>
-      <x:c r="E15" s="66"/>
-      <x:c r="F15" s="66"/>
+      <x:c r="A15" s="67"/>
+      <x:c r="B15" s="67"/>
+      <x:c r="C15" s="67"/>
+      <x:c r="D15" s="67"/>
+      <x:c r="E15" s="67"/>
+      <x:c r="F15" s="67"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="50" t="str">
         <x:v>OVERALL</x:v>
       </x:c>
       <x:c r="B16" s="50" t="str">
-        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
+        <x:v>CASCADE_CONTRACT_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C16" s="50"/>
       <x:c r="D16" s="50"/>
       <x:c r="E16" s="50"/>
       <x:c r="F16" s="50" t="str">
-        <x:v>Atlanta player-game and competitive-stint outcomes remain</x:v>
+        <x:v>Atlanta player-game and above-baseline competitive stints remain</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11772,7 +12582,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -12061,7 +12871,7 @@
         <x:v>Nuggets — Thomas Welsh two-way</x:v>
       </x:c>
       <x:c r="C23" s="51" t="str">
-        <x:v>Actual Welsh two-way destination used as role-preservation baseline</x:v>
+        <x:v>Actual Welsh occupied one Denver two-way slot</x:v>
       </x:c>
       <x:c r="D23" s="51" t="str">
         <x:v>https://www.nba.com/nuggets/news/thomas-welsh-signs-two-way-contract-071918</x:v>
@@ -12177,6 +12987,174 @@
       </x:c>
       <x:c r="D31" s="51" t="str">
         <x:v>https://www.nba.com/spurs/news/san-antonio-assigns-chimezie-metu-austin-spurs-8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="51" t="str">
+        <x:v>S28</x:v>
+      </x:c>
+      <x:c r="B32" s="51" t="str">
+        <x:v>Mavericks — Spalding signing</x:v>
+      </x:c>
+      <x:c r="C32" s="51" t="str">
+        <x:v>Dallas signed the actual #56 pick to a standard NBA contract</x:v>
+      </x:c>
+      <x:c r="D32" s="51" t="str">
+        <x:v>https://www.nba.com/mavs/mavericks-sign-forward-ray-spalding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="51" t="str">
+        <x:v>S29</x:v>
+      </x:c>
+      <x:c r="B33" s="51" t="str">
+        <x:v>Mavericks — Porzingis trade and Spalding waiver</x:v>
+      </x:c>
+      <x:c r="C33" s="51" t="str">
+        <x:v>Spalding appeared in one Dallas game and was waived in the Jan. 31 roster move</x:v>
+      </x:c>
+      <x:c r="D33" s="51" t="str">
+        <x:v>https://www.nba.com/mavs/mavericks-acquire-all-star-kristaps-porzingis-tim-hardaway-jr-courtney-lee-and-trey-burke-in-trade-with-knicks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="51" t="str">
+        <x:v>S30</x:v>
+      </x:c>
+      <x:c r="B34" s="51" t="str">
+        <x:v>NBA G League — Ray Spalding</x:v>
+      </x:c>
+      <x:c r="C34" s="51" t="str">
+        <x:v>2018-19 Texas: 29 games, 26 starts, 30.1 MPG</x:v>
+      </x:c>
+      <x:c r="D34" s="51" t="str">
+        <x:v>https://gleague.nba.com/player/1629034/ray-spalding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="51" t="str">
+        <x:v>S31</x:v>
+      </x:c>
+      <x:c r="B35" s="51" t="str">
+        <x:v>Nuggets — Thomas Welsh two-way</x:v>
+      </x:c>
+      <x:c r="C35" s="51" t="str">
+        <x:v>Denver signed the actual #58 pick to a two-way contract</x:v>
+      </x:c>
+      <x:c r="D35" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/thomas-welsh-signs-two-way-contract-071918</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="51" t="str">
+        <x:v>S32</x:v>
+      </x:c>
+      <x:c r="B36" s="51" t="str">
+        <x:v>Nuggets — 2018-19 two-way preview</x:v>
+      </x:c>
+      <x:c r="C36" s="51" t="str">
+        <x:v>Welsh and Akoon-Purcell occupied Denver's two two-way positions</x:v>
+      </x:c>
+      <x:c r="D36" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/1819-player-previews-akoon-purcell-welsh-091918</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="51" t="str">
+        <x:v>S33</x:v>
+      </x:c>
+      <x:c r="B37" s="51" t="str">
+        <x:v>NBA G League — 2018 two-way rule</x:v>
+      </x:c>
+      <x:c r="C37" s="51" t="str">
+        <x:v>2018-19 teams could carry two two-way players beyond the 15-man roster</x:v>
+      </x:c>
+      <x:c r="D37" s="51" t="str">
+        <x:v>https://windycity.gleague.nba.com/news/bulls-sign-brandon-sampson-to-two-way-contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="51" t="str">
+        <x:v>S34</x:v>
+      </x:c>
+      <x:c r="B38" s="51" t="str">
+        <x:v>Nuggets — Welsh 2018-19 recap</x:v>
+      </x:c>
+      <x:c r="C38" s="51" t="str">
+        <x:v>Welsh played 11 NBA games and 36 minutes; G League was his primary venue</x:v>
+      </x:c>
+      <x:c r="D38" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/denver-nuggets-thomas-welsh-excited-for-nba-summer-league-070219c</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="51" t="str">
+        <x:v>S35</x:v>
+      </x:c>
+      <x:c r="B39" s="51" t="str">
+        <x:v>RealGM — Thomas Welsh profile</x:v>
+      </x:c>
+      <x:c r="C39" s="51" t="str">
+        <x:v>Two-way transaction and 20-game G League allocation baseline</x:v>
+      </x:c>
+      <x:c r="D39" s="51" t="str">
+        <x:v>https://basketball.realgm.com/player/Thomas-Welsh/Summary/64323</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="51" t="str">
+        <x:v>S36</x:v>
+      </x:c>
+      <x:c r="B40" s="51" t="str">
+        <x:v>NBA — 2018-11-15 Atlanta at Denver</x:v>
+      </x:c>
+      <x:c r="C40" s="51" t="str">
+        <x:v>Denver 138-93 official game baseline</x:v>
+      </x:c>
+      <x:c r="D40" s="51" t="str">
+        <x:v>https://www.nba.com/game/atl-vs-den-0021800214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="51" t="str">
+        <x:v>S37</x:v>
+      </x:c>
+      <x:c r="B41" s="51" t="str">
+        <x:v>Basketball-Reference — 2018-11-15 box score</x:v>
+      </x:c>
+      <x:c r="C41" s="51" t="str">
+        <x:v>Welsh did not play against Atlanta</x:v>
+      </x:c>
+      <x:c r="D41" s="51" t="str">
+        <x:v>https://www.basketball-reference.com/boxscores/201811150DEN.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="51" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="B42" s="51" t="str">
+        <x:v>NBA Hawks — 2018-12-08 Denver at Atlanta</x:v>
+      </x:c>
+      <x:c r="C42" s="51" t="str">
+        <x:v>Atlanta 106-98 official game baseline</x:v>
+      </x:c>
+      <x:c r="D42" s="51" t="str">
+        <x:v>https://www.nba.com/hawks/game/0021800380</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="51" t="str">
+        <x:v>S39</x:v>
+      </x:c>
+      <x:c r="B43" s="51" t="str">
+        <x:v>Basketball-Reference — 2018-12-08 box score</x:v>
+      </x:c>
+      <x:c r="C43" s="51" t="str">
+        <x:v>Welsh did not play against Atlanta</x:v>
+      </x:c>
+      <x:c r="D43" s="51" t="str">
+        <x:v>https://www.basketball-reference.com/boxscores/201812080ATL.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12185,7 +13163,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c25f5cf78044f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52b7422b3c84448d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Close Dallas and Denver cascade contract layers (#38)
Close the downstream contract-layer cascade from the 2018 #30 counterfactual while preserving team-specific rookie roles and keeping game outcomes on hold.
</commit_message>
<xml_diff>
--- a/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
+++ b/simulation/ATLANTA_2018_19_CAUSALITY_LEDGER.xlsx
@@ -2,14 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R366e1f9bc1784d4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="Rac03984f160d43c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="Ra5b04d9f3a924551"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R3e5d45d21e1545b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurs Impact" sheetId="5" r:id="R60f9cfc284d9453b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="6" r:id="Ra11d836a74e4428d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="7" r:id="Rc70dc5e77334451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="8" r:id="R342fc8719a2a4474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R68f787c966524bf9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Game Ledger" sheetId="2" r:id="R0da9e4168273453e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Season Minutes" sheetId="3" r:id="R9235d60d1db24783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2018 Draft Board" sheetId="4" r:id="R66f8d0ab790c4c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Spurs Impact" sheetId="5" r:id="R30ddbd1fb9b245ff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cascade Impact" sheetId="6" r:id="Rc3254edf00a34c83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Draft Bridge" sheetId="7" r:id="R880401c26dbd44e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Gate Audit" sheetId="8" r:id="Rc96c56130c3c4d65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="9" r:id="R5bb35b2c8e9a47f0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -182,7 +183,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="67">
+  <x:cellXfs count="68">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -309,6 +310,9 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="10" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="203" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
@@ -437,7 +441,48 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SourceTable" displayName="SourceTable" ref="A4:D31" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="CascadeContractTable" displayName="CascadeContractTable" ref="A6:M12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="13">
+    <x:tableColumn id="1" name="Team"/>
+    <x:tableColumn id="2" name="World"/>
+    <x:tableColumn id="3" name="Player"/>
+    <x:tableColumn id="4" name="Pick"/>
+    <x:tableColumn id="5" name="Contract layer"/>
+    <x:tableColumn id="6" name="Development path"/>
+    <x:tableColumn id="7" name="NBA GP"/>
+    <x:tableColumn id="8" name="NBA MIN"/>
+    <x:tableColumn id="9" name="G League GP"/>
+    <x:tableColumn id="10" name="Transaction"/>
+    <x:tableColumn id="11" name="Role status"/>
+    <x:tableColumn id="12" name="Escalation trigger"/>
+    <x:tableColumn id="13" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="CascadeDirectGameTable" displayName="CascadeDirectGameTable" ref="A15:L19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="12">
+    <x:tableColumn id="1" name="Team"/>
+    <x:tableColumn id="2" name="Date"/>
+    <x:tableColumn id="3" name="Site"/>
+    <x:tableColumn id="4" name="Actual"/>
+    <x:tableColumn id="5" name="Team pts"/>
+    <x:tableColumn id="6" name="ATL pts"/>
+    <x:tableColumn id="7" name="Margin"/>
+    <x:tableColumn id="8" name="Replaced player"/>
+    <x:tableColumn id="9" name="Replaced MIN"/>
+    <x:tableColumn id="10" name="CF contact"/>
+    <x:tableColumn id="11" name="Outcome status"/>
+    <x:tableColumn id="12" name="Source ID"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="SourceTable" displayName="SourceTable" ref="A4:D43" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="4">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="Source"/>
@@ -655,7 +700,7 @@
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
       <x:c r="A1" s="18" t="str">
-        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.3</x:v>
+        <x:v>ATLANTA 2018-19 — CAUSALITY LEDGER / DRAFT BOARD v0.4</x:v>
       </x:c>
       <x:c r="B1" s="19"/>
       <x:c r="C1" s="19"/>
@@ -690,13 +735,13 @@
         <x:v>Status</x:v>
       </x:c>
       <x:c r="B4" s="20" t="str">
-        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
+        <x:v>CASCADE_CONTRACT_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C4" s="20" t="str">
         <x:v>Canon</x:v>
       </x:c>
       <x:c r="D4" s="20" t="str">
-        <x:v>PROVISIONAL</x:v>
+        <x:v>v0.22 PARTIAL</x:v>
       </x:c>
       <x:c r="E4" s="20" t="str">
         <x:v>Manuscript</x:v>
@@ -990,7 +1035,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B18" s="22" t="str">
-        <x:v>Spellman's San Antonio #49 baseline role is closed at Metu's low-leverage slot. Any minutes above 145.4 need a dated donor; competitive stints trigger outcome review.</x:v>
+        <x:v>The San Antonio, Dallas, and Denver replacement contract layers are closed. Each CF rookie starts inside the displaced player's team-specific role, not his old-team minutes.</x:v>
       </x:c>
       <x:c r="C18" s="22"/>
       <x:c r="D18" s="22"/>
@@ -1004,7 +1049,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B19" s="22" t="str">
-        <x:v>No counterfactual scores or results have been generated. Manual flips and close-game cherry-picking are prohibited.</x:v>
+        <x:v>Welsh cannot duplicate Denver's occupied two-way slot. His undrafted free-agent destination remains HOLD; no counterfactual scores or results have been generated.</x:v>
       </x:c>
       <x:c r="C19" s="22"/>
       <x:c r="D19" s="22"/>
@@ -8062,7 +8107,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R70e1b02e502342a0"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2a1e5b9d80d449ee"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9101,7 +9146,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0edad3bb7357419f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d537aa0b8ad4ad9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -9154,7 +9199,7 @@
         <x:v>Next blocker</x:v>
       </x:c>
       <x:c r="H4" s="6" t="str">
-        <x:v>Dallas/Denver contracts</x:v>
+        <x:v>Atlanta donor vector</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -10131,10 +10176,10 @@
         <x:v>Metu is the displaced #49 athletic big and remains above this slot.</x:v>
       </x:c>
       <x:c r="J33" s="53" t="str">
-        <x:v>Dallas role/minutes HOLD</x:v>
+        <x:v>Dallas contract layer PASS; outcomes HOLD</x:v>
       </x:c>
       <x:c r="K33" s="53" t="str">
-        <x:v>S13/S15</x:v>
+        <x:v>S13/S15/S28/S29/S30</x:v>
       </x:c>
     </x:row>
     <x:row r="34">
@@ -10201,10 +10246,10 @@
         <x:v>Spalding was graded in the drafted second-round big tier.</x:v>
       </x:c>
       <x:c r="J35" s="53" t="str">
-        <x:v>Denver role/two-way HOLD</x:v>
+        <x:v>Denver contract layer PASS; Welsh market HOLD</x:v>
       </x:c>
       <x:c r="K35" s="53" t="str">
-        <x:v>S18</x:v>
+        <x:v>S18/S31/S32/S33/S34</x:v>
       </x:c>
     </x:row>
     <x:row r="36">
@@ -10283,7 +10328,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb23b2dbd43ef4286"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc6d353ac21e5413d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -11288,12 +11333,777 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R678b9e0485934009"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5c86b37a184f22"/>
   </x:tableParts>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="16" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="23" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="25" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="25" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="16" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="16" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="25" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="46" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="18" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="32" customHeight="1">
+      <x:c r="A1" s="3" t="str">
+        <x:v>DALLAS / DENVER 2018-19 — CASCADE CONTRACT FIREWALL</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="56" t="str">
+        <x:v>Dallas base</x:v>
+      </x:c>
+      <x:c r="B4" s="56" t="str">
+        <x:v>1 G / 1 MIN</x:v>
+      </x:c>
+      <x:c r="C4" s="56"/>
+      <x:c r="D4" s="56" t="str">
+        <x:v>Texas</x:v>
+      </x:c>
+      <x:c r="E4" s="56" t="str">
+        <x:v>29 G / 30.1 MPG</x:v>
+      </x:c>
+      <x:c r="F4" s="56"/>
+      <x:c r="G4" s="56" t="str">
+        <x:v>Denver base</x:v>
+      </x:c>
+      <x:c r="H4" s="56" t="str">
+        <x:v>11 G / 36 MIN</x:v>
+      </x:c>
+      <x:c r="I4" s="56"/>
+      <x:c r="J4" s="56" t="str">
+        <x:v>ATL series</x:v>
+      </x:c>
+      <x:c r="K4" s="56" t="str">
+        <x:v>4 G / 0 MIN</x:v>
+      </x:c>
+      <x:c r="L4" s="56" t="str">
+        <x:v>Status</x:v>
+      </x:c>
+      <x:c r="M4" s="56" t="str">
+        <x:v>CONTRACT_LAYER_PASS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="57"/>
+      <x:c r="B5" s="57"/>
+      <x:c r="C5" s="57"/>
+      <x:c r="D5" s="57"/>
+      <x:c r="E5" s="57"/>
+      <x:c r="F5" s="57"/>
+      <x:c r="G5" s="57"/>
+      <x:c r="H5" s="57"/>
+      <x:c r="I5" s="57"/>
+      <x:c r="J5" s="57"/>
+      <x:c r="K5" s="57"/>
+      <x:c r="L5" s="57"/>
+      <x:c r="M5" s="57"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="40" t="str">
+        <x:v>Team</x:v>
+      </x:c>
+      <x:c r="B6" s="40" t="str">
+        <x:v>World</x:v>
+      </x:c>
+      <x:c r="C6" s="40" t="str">
+        <x:v>Player</x:v>
+      </x:c>
+      <x:c r="D6" s="40" t="str">
+        <x:v>Pick</x:v>
+      </x:c>
+      <x:c r="E6" s="40" t="str">
+        <x:v>Contract layer</x:v>
+      </x:c>
+      <x:c r="F6" s="40" t="str">
+        <x:v>Development path</x:v>
+      </x:c>
+      <x:c r="G6" s="40" t="str">
+        <x:v>NBA GP</x:v>
+      </x:c>
+      <x:c r="H6" s="40" t="str">
+        <x:v>NBA MIN</x:v>
+      </x:c>
+      <x:c r="I6" s="40" t="str">
+        <x:v>G League GP</x:v>
+      </x:c>
+      <x:c r="J6" s="40" t="str">
+        <x:v>Transaction</x:v>
+      </x:c>
+      <x:c r="K6" s="40" t="str">
+        <x:v>Role status</x:v>
+      </x:c>
+      <x:c r="L6" s="40" t="str">
+        <x:v>Escalation trigger</x:v>
+      </x:c>
+      <x:c r="M6" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="61" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B7" s="61" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="C7" s="61" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="D7" s="61" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E7" s="61" t="str">
+        <x:v>Standard NBA</x:v>
+      </x:c>
+      <x:c r="F7" s="61" t="str">
+        <x:v>Texas assignment</x:v>
+      </x:c>
+      <x:c r="G7" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H7" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I7" s="61" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J7" s="61" t="str">
+        <x:v>Waived 2019-01-31</x:v>
+      </x:c>
+      <x:c r="K7" s="61" t="str">
+        <x:v>ACTUAL_REPLACED</x:v>
+      </x:c>
+      <x:c r="L7" s="61" t="str">
+        <x:v>Reference only</x:v>
+      </x:c>
+      <x:c r="M7" s="61" t="str">
+        <x:v>S28/S29/S30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="61" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B8" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C8" s="61" t="str">
+        <x:v>Chimezie Metu</x:v>
+      </x:c>
+      <x:c r="D8" s="61" t="n">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="E8" s="61" t="str">
+        <x:v>Standard NBA layer</x:v>
+      </x:c>
+      <x:c r="F8" s="61" t="str">
+        <x:v>Texas assignment baseline</x:v>
+      </x:c>
+      <x:c r="G8" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H8" s="61" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="I8" s="61" t="n">
+        <x:v>29</x:v>
+      </x:c>
+      <x:c r="J8" s="61" t="str">
+        <x:v>Jan. 31 waiver choice HOLD</x:v>
+      </x:c>
+      <x:c r="K8" s="61" t="str">
+        <x:v>CF_CHANGED_STANDARD</x:v>
+      </x:c>
+      <x:c r="L8" s="61" t="str">
+        <x:v>&gt;1 NBA MIN or a different waiver opens Dallas player-game review</x:v>
+      </x:c>
+      <x:c r="M8" s="61" t="str">
+        <x:v>S28/S29/S30</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B9" s="61" t="str">
+        <x:v>ACTUAL</x:v>
+      </x:c>
+      <x:c r="C9" s="61" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="D9" s="61" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E9" s="61" t="str">
+        <x:v>Two-way</x:v>
+      </x:c>
+      <x:c r="F9" s="61" t="str">
+        <x:v>Capital City / Iowa</x:v>
+      </x:c>
+      <x:c r="G9" s="61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H9" s="61" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I9" s="61" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J9" s="61" t="str">
+        <x:v>Two-way ended 2019-07-30</x:v>
+      </x:c>
+      <x:c r="K9" s="61" t="str">
+        <x:v>ACTUAL_REPLACED</x:v>
+      </x:c>
+      <x:c r="L9" s="61" t="str">
+        <x:v>Reference only</x:v>
+      </x:c>
+      <x:c r="M9" s="61" t="str">
+        <x:v>S31/S34/S35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B10" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C10" s="61" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="D10" s="61" t="n">
+        <x:v>58</x:v>
+      </x:c>
+      <x:c r="E10" s="61" t="str">
+        <x:v>Two-way (Welsh slot)</x:v>
+      </x:c>
+      <x:c r="F10" s="61" t="str">
+        <x:v>External G League assignment class</x:v>
+      </x:c>
+      <x:c r="G10" s="61" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="H10" s="61" t="n">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="I10" s="61" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="J10" s="61" t="str">
+        <x:v>Season role baseline</x:v>
+      </x:c>
+      <x:c r="K10" s="61" t="str">
+        <x:v>CF_CHANGED_TWO_WAY</x:v>
+      </x:c>
+      <x:c r="L10" s="61" t="str">
+        <x:v>&gt;36 NBA MIN or different dates opens Denver player-game review</x:v>
+      </x:c>
+      <x:c r="M10" s="61" t="str">
+        <x:v>S31/S32/S33/S34</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B11" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C11" s="61" t="str">
+        <x:v>DeVaughn Akoon-Purcell</x:v>
+      </x:c>
+      <x:c r="D11" s="61"/>
+      <x:c r="E11" s="61" t="str">
+        <x:v>Two-way</x:v>
+      </x:c>
+      <x:c r="F11" s="61" t="str">
+        <x:v>G League development</x:v>
+      </x:c>
+      <x:c r="G11" s="61"/>
+      <x:c r="H11" s="61"/>
+      <x:c r="I11" s="61"/>
+      <x:c r="J11" s="61" t="str">
+        <x:v>Actual second slot preserved</x:v>
+      </x:c>
+      <x:c r="K11" s="61" t="str">
+        <x:v>CF_PROTECTED_TWO_WAY</x:v>
+      </x:c>
+      <x:c r="L11" s="61" t="str">
+        <x:v>Do not displace without a new transaction cause</x:v>
+      </x:c>
+      <x:c r="M11" s="61" t="str">
+        <x:v>S32/S33</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="61" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B12" s="61" t="str">
+        <x:v>CF</x:v>
+      </x:c>
+      <x:c r="C12" s="61" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="D12" s="61"/>
+      <x:c r="E12" s="61" t="str">
+        <x:v>No Denver slot</x:v>
+      </x:c>
+      <x:c r="F12" s="61" t="str">
+        <x:v>Undrafted free-agent market</x:v>
+      </x:c>
+      <x:c r="G12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="H12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="61" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="61" t="str">
+        <x:v>Destination unresolved</x:v>
+      </x:c>
+      <x:c r="K12" s="61" t="str">
+        <x:v>CF_OUT_NO_SLOT</x:v>
+      </x:c>
+      <x:c r="L12" s="61" t="str">
+        <x:v>Any NBA signing creates a new team-impact branch</x:v>
+      </x:c>
+      <x:c r="M12" s="61" t="str">
+        <x:v>S31/S32/S33/S35</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="57"/>
+      <x:c r="B13" s="57"/>
+      <x:c r="C13" s="57"/>
+      <x:c r="D13" s="57"/>
+      <x:c r="E13" s="57"/>
+      <x:c r="F13" s="57"/>
+      <x:c r="G13" s="57"/>
+      <x:c r="H13" s="57"/>
+      <x:c r="I13" s="57"/>
+      <x:c r="J13" s="57"/>
+      <x:c r="K13" s="57"/>
+      <x:c r="L13" s="57"/>
+      <x:c r="M13" s="57"/>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="57"/>
+      <x:c r="B14" s="57"/>
+      <x:c r="C14" s="57"/>
+      <x:c r="D14" s="57"/>
+      <x:c r="E14" s="57"/>
+      <x:c r="F14" s="57"/>
+      <x:c r="G14" s="57"/>
+      <x:c r="H14" s="57"/>
+      <x:c r="I14" s="57"/>
+      <x:c r="J14" s="57"/>
+      <x:c r="K14" s="57"/>
+      <x:c r="L14" s="57"/>
+      <x:c r="M14" s="57"/>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="40" t="str">
+        <x:v>Team</x:v>
+      </x:c>
+      <x:c r="B15" s="40" t="str">
+        <x:v>Date</x:v>
+      </x:c>
+      <x:c r="C15" s="40" t="str">
+        <x:v>Site</x:v>
+      </x:c>
+      <x:c r="D15" s="40" t="str">
+        <x:v>Actual</x:v>
+      </x:c>
+      <x:c r="E15" s="40" t="str">
+        <x:v>Team pts</x:v>
+      </x:c>
+      <x:c r="F15" s="40" t="str">
+        <x:v>ATL pts</x:v>
+      </x:c>
+      <x:c r="G15" s="40" t="str">
+        <x:v>Margin</x:v>
+      </x:c>
+      <x:c r="H15" s="40" t="str">
+        <x:v>Replaced player</x:v>
+      </x:c>
+      <x:c r="I15" s="40" t="str">
+        <x:v>Replaced MIN</x:v>
+      </x:c>
+      <x:c r="J15" s="40" t="str">
+        <x:v>CF contact</x:v>
+      </x:c>
+      <x:c r="K15" s="40" t="str">
+        <x:v>Outcome status</x:v>
+      </x:c>
+      <x:c r="L15" s="40" t="str">
+        <x:v>Source ID</x:v>
+      </x:c>
+      <x:c r="M15" s="57"/>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="58" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B16" s="59" t="n">
+        <x:v>43397.5</x:v>
+      </x:c>
+      <x:c r="C16" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D16" s="58" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E16" s="58" t="n">
+        <x:v>104</x:v>
+      </x:c>
+      <x:c r="F16" s="58" t="n">
+        <x:v>111</x:v>
+      </x:c>
+      <x:c r="G16" s="58" t="n">
+        <x:v>-7</x:v>
+      </x:c>
+      <x:c r="H16" s="58" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="I16" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J16" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K16" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L16" s="58" t="str">
+        <x:v>S10/S29</x:v>
+      </x:c>
+      <x:c r="M16" s="57"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="58" t="str">
+        <x:v>Dallas</x:v>
+      </x:c>
+      <x:c r="B17" s="59" t="n">
+        <x:v>43446.5</x:v>
+      </x:c>
+      <x:c r="C17" s="58" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D17" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E17" s="58" t="n">
+        <x:v>114</x:v>
+      </x:c>
+      <x:c r="F17" s="58" t="n">
+        <x:v>107</x:v>
+      </x:c>
+      <x:c r="G17" s="58" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="H17" s="58" t="str">
+        <x:v>Ray Spalding</x:v>
+      </x:c>
+      <x:c r="I17" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K17" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L17" s="58" t="str">
+        <x:v>S11/S29</x:v>
+      </x:c>
+      <x:c r="M17" s="57"/>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="58" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B18" s="59" t="n">
+        <x:v>43419.5</x:v>
+      </x:c>
+      <x:c r="C18" s="58" t="str">
+        <x:v>H</x:v>
+      </x:c>
+      <x:c r="D18" s="58" t="str">
+        <x:v>W</x:v>
+      </x:c>
+      <x:c r="E18" s="58" t="n">
+        <x:v>138</x:v>
+      </x:c>
+      <x:c r="F18" s="58" t="n">
+        <x:v>93</x:v>
+      </x:c>
+      <x:c r="G18" s="58" t="n">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="H18" s="58" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="I18" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J18" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K18" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L18" s="58" t="str">
+        <x:v>S36/S37</x:v>
+      </x:c>
+      <x:c r="M18" s="57"/>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="58" t="str">
+        <x:v>Denver</x:v>
+      </x:c>
+      <x:c r="B19" s="59" t="n">
+        <x:v>43442.5</x:v>
+      </x:c>
+      <x:c r="C19" s="58" t="str">
+        <x:v>A</x:v>
+      </x:c>
+      <x:c r="D19" s="58" t="str">
+        <x:v>L</x:v>
+      </x:c>
+      <x:c r="E19" s="58" t="n">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="F19" s="58" t="n">
+        <x:v>106</x:v>
+      </x:c>
+      <x:c r="G19" s="58" t="n">
+        <x:v>-8</x:v>
+      </x:c>
+      <x:c r="H19" s="58" t="str">
+        <x:v>Thomas Welsh</x:v>
+      </x:c>
+      <x:c r="I19" s="58" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J19" s="58" t="str">
+        <x:v>NO_DIRECT_MINUTES</x:v>
+      </x:c>
+      <x:c r="K19" s="58" t="str">
+        <x:v>ATL-side execution HOLD</x:v>
+      </x:c>
+      <x:c r="L19" s="58" t="str">
+        <x:v>S38/S39</x:v>
+      </x:c>
+      <x:c r="M19" s="57"/>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="57"/>
+      <x:c r="B20" s="57"/>
+      <x:c r="C20" s="57"/>
+      <x:c r="D20" s="57"/>
+      <x:c r="E20" s="57"/>
+      <x:c r="F20" s="57"/>
+      <x:c r="G20" s="57"/>
+      <x:c r="H20" s="57"/>
+      <x:c r="I20" s="57"/>
+      <x:c r="J20" s="57"/>
+      <x:c r="K20" s="57"/>
+      <x:c r="L20" s="57"/>
+      <x:c r="M20" s="57"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="60" t="str">
+        <x:v>Dallas: Metu begins inside Spalding's standard-contract / Texas assignment slot; a different Jan. 31 waiver choice remains HOLD. Denver: Spalding takes Welsh's two-way slot, Akoon-Purcell keeps the other, and Welsh moves to the undrafted free-agent market. Any minutes above the displaced-player base reopen player-game review.</x:v>
+      </x:c>
+      <x:c r="B21" s="60"/>
+      <x:c r="C21" s="60"/>
+      <x:c r="D21" s="60"/>
+      <x:c r="E21" s="60"/>
+      <x:c r="F21" s="60"/>
+      <x:c r="G21" s="60"/>
+      <x:c r="H21" s="60"/>
+      <x:c r="I21" s="57"/>
+      <x:c r="J21" s="40" t="str">
+        <x:v>Audit</x:v>
+      </x:c>
+      <x:c r="K21" s="40" t="str">
+        <x:v>Value</x:v>
+      </x:c>
+      <x:c r="L21" s="40" t="str">
+        <x:v>Check</x:v>
+      </x:c>
+      <x:c r="M21" s="57"/>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="60"/>
+      <x:c r="B22" s="60"/>
+      <x:c r="C22" s="60"/>
+      <x:c r="D22" s="60"/>
+      <x:c r="E22" s="60"/>
+      <x:c r="F22" s="60"/>
+      <x:c r="G22" s="60"/>
+      <x:c r="H22" s="60"/>
+      <x:c r="I22" s="57"/>
+      <x:c r="J22" s="58" t="str">
+        <x:v>Changed contract chains</x:v>
+      </x:c>
+      <x:c r="K22" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_CHANGED_STANDARD")+COUNTIF(K7:K12,"CF_CHANGED_TWO_WAY")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L22" s="58" t="str">
+        <x:f>IF(K22=2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M22" s="57"/>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="60"/>
+      <x:c r="B23" s="60"/>
+      <x:c r="C23" s="60"/>
+      <x:c r="D23" s="60"/>
+      <x:c r="E23" s="60"/>
+      <x:c r="F23" s="60"/>
+      <x:c r="G23" s="60"/>
+      <x:c r="H23" s="60"/>
+      <x:c r="I23" s="57"/>
+      <x:c r="J23" s="58" t="str">
+        <x:v>Direct games</x:v>
+      </x:c>
+      <x:c r="K23" s="58" t="n">
+        <x:f>COUNTA(A16:A19)</x:f>
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="L23" s="58" t="str">
+        <x:f>IF(K23=4,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M23" s="57"/>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="57"/>
+      <x:c r="B24" s="57"/>
+      <x:c r="C24" s="57"/>
+      <x:c r="D24" s="57"/>
+      <x:c r="E24" s="57"/>
+      <x:c r="F24" s="57"/>
+      <x:c r="G24" s="57"/>
+      <x:c r="H24" s="57"/>
+      <x:c r="I24" s="57"/>
+      <x:c r="J24" s="58" t="str">
+        <x:v>Direct replaced minutes</x:v>
+      </x:c>
+      <x:c r="K24" s="58" t="n">
+        <x:f>SUM(I16:I19)</x:f>
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L24" s="58" t="str">
+        <x:f>IF(K24=0,"PASS","REVIEW")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M24" s="57"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="57"/>
+      <x:c r="B25" s="57"/>
+      <x:c r="C25" s="57"/>
+      <x:c r="D25" s="57"/>
+      <x:c r="E25" s="57"/>
+      <x:c r="F25" s="57"/>
+      <x:c r="G25" s="57"/>
+      <x:c r="H25" s="57"/>
+      <x:c r="I25" s="57"/>
+      <x:c r="J25" s="58" t="str">
+        <x:v>Denver CF two-way slots</x:v>
+      </x:c>
+      <x:c r="K25" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_CHANGED_TWO_WAY")+COUNTIF(K7:K12,"CF_PROTECTED_TWO_WAY")</x:f>
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="L25" s="58" t="str">
+        <x:f>IF(K25=2,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M25" s="57"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="57"/>
+      <x:c r="B26" s="57"/>
+      <x:c r="C26" s="57"/>
+      <x:c r="D26" s="57"/>
+      <x:c r="E26" s="57"/>
+      <x:c r="F26" s="57"/>
+      <x:c r="G26" s="57"/>
+      <x:c r="H26" s="57"/>
+      <x:c r="I26" s="57"/>
+      <x:c r="J26" s="58" t="str">
+        <x:v>Welsh duplicate blocked</x:v>
+      </x:c>
+      <x:c r="K26" s="58" t="n">
+        <x:f>COUNTIF(K7:K12,"CF_OUT_NO_SLOT")</x:f>
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="L26" s="58" t="str">
+        <x:f>IF(K26=1,"PASS","FAIL")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M26" s="57"/>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="57"/>
+      <x:c r="B27" s="57"/>
+      <x:c r="C27" s="57"/>
+      <x:c r="D27" s="57"/>
+      <x:c r="E27" s="57"/>
+      <x:c r="F27" s="57"/>
+      <x:c r="G27" s="57"/>
+      <x:c r="H27" s="57"/>
+      <x:c r="I27" s="57"/>
+      <x:c r="J27" s="58" t="str">
+        <x:v>Outcome lock</x:v>
+      </x:c>
+      <x:c r="K27" s="58" t="str">
+        <x:f>IF(AND(K24=0,K25=2,K26=1),"CASCADE DIRECT PASS","REVIEW")</x:f>
+        <x:v>CASCADE DIRECT PASS</x:v>
+      </x:c>
+      <x:c r="L27" s="58" t="str">
+        <x:f>IF(K27="CASCADE DIRECT PASS","PASS","HOLD")</x:f>
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="M27" s="57"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:M2"/>
+    <x:mergeCell ref="A21:H23"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="2">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rebf6d880b3174b0b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2d3711a7d9ae4c67"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -11359,10 +12169,10 @@
       <x:c r="D5" s="13" t="n">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="E5" s="61" t="n">
+      <x:c r="E5" s="62" t="n">
         <x:v>0.105</x:v>
       </x:c>
-      <x:c r="F5" s="61" t="n">
+      <x:c r="F5" s="62" t="n">
         <x:v>0.4212</x:v>
       </x:c>
       <x:c r="G5" s="13" t="n">
@@ -11391,10 +12201,10 @@
       <x:c r="D6" s="13" t="n">
         <x:v>9</x:v>
       </x:c>
-      <x:c r="E6" s="61" t="n">
+      <x:c r="E6" s="62" t="n">
         <x:v>0.06</x:v>
       </x:c>
-      <x:c r="F6" s="61" t="n">
+      <x:c r="F6" s="62" t="n">
         <x:v>0.263</x:v>
       </x:c>
       <x:c r="G6" s="13" t="n">
@@ -11490,8 +12300,8 @@
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="64" t="str">
-        <x:v>FINAL BLOCKER: Spurs baseline role is closed. Execute Atlanta player-game impacts and review any Spellman competitive stints before standings/lottery.</x:v>
+      <x:c r="A14" s="65" t="str">
+        <x:v>FINAL BLOCKER: Spurs, Dallas, and Denver contract layers are closed. Execute Atlanta player-game impacts and review only minutes beyond each displaced-player base before standings/lottery.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11505,7 +12315,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -11547,10 +12357,10 @@
         <x:v>G0</x:v>
       </x:c>
       <x:c r="B5" s="51" t="str">
-        <x:v>Spellman destination + second-team baseline</x:v>
+        <x:v>Changed-pick contract and direct-game baselines</x:v>
       </x:c>
       <x:c r="C5" s="51" t="str">
-        <x:v>Spurs #49; base 29 G/145.4 min; ATL series 0 min</x:v>
+        <x:v>Spurs 145.4 min; Dallas 1 min; Denver 36 min; ATL series all 0</x:v>
       </x:c>
       <x:c r="D5" s="53" t="str">
         <x:v>PASS</x:v>
@@ -11559,7 +12369,7 @@
         <x:v>None</x:v>
       </x:c>
       <x:c r="F5" s="51" t="str">
-        <x:v>Preserve role cap and donor trigger</x:v>
+        <x:v>Preserve team-specific caps and triggers</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -11743,25 +12553,25 @@
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="66"/>
-      <x:c r="B15" s="66"/>
-      <x:c r="C15" s="66"/>
-      <x:c r="D15" s="66"/>
-      <x:c r="E15" s="66"/>
-      <x:c r="F15" s="66"/>
+      <x:c r="A15" s="67"/>
+      <x:c r="B15" s="67"/>
+      <x:c r="C15" s="67"/>
+      <x:c r="D15" s="67"/>
+      <x:c r="E15" s="67"/>
+      <x:c r="F15" s="67"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="50" t="str">
         <x:v>OVERALL</x:v>
       </x:c>
       <x:c r="B16" s="50" t="str">
-        <x:v>SECOND_TEAM_BASELINE_PASS / OUTCOME_HOLD</x:v>
+        <x:v>CASCADE_CONTRACT_PASS / OUTCOME_HOLD</x:v>
       </x:c>
       <x:c r="C16" s="50"/>
       <x:c r="D16" s="50"/>
       <x:c r="E16" s="50"/>
       <x:c r="F16" s="50" t="str">
-        <x:v>Atlanta player-game and competitive-stint outcomes remain</x:v>
+        <x:v>Atlanta player-game and above-baseline competitive stints remain</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11772,7 +12582,7 @@
 </x:worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
@@ -12061,7 +12871,7 @@
         <x:v>Nuggets — Thomas Welsh two-way</x:v>
       </x:c>
       <x:c r="C23" s="51" t="str">
-        <x:v>Actual Welsh two-way destination used as role-preservation baseline</x:v>
+        <x:v>Actual Welsh occupied one Denver two-way slot</x:v>
       </x:c>
       <x:c r="D23" s="51" t="str">
         <x:v>https://www.nba.com/nuggets/news/thomas-welsh-signs-two-way-contract-071918</x:v>
@@ -12177,6 +12987,174 @@
       </x:c>
       <x:c r="D31" s="51" t="str">
         <x:v>https://www.nba.com/spurs/news/san-antonio-assigns-chimezie-metu-austin-spurs-8</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="51" t="str">
+        <x:v>S28</x:v>
+      </x:c>
+      <x:c r="B32" s="51" t="str">
+        <x:v>Mavericks — Spalding signing</x:v>
+      </x:c>
+      <x:c r="C32" s="51" t="str">
+        <x:v>Dallas signed the actual #56 pick to a standard NBA contract</x:v>
+      </x:c>
+      <x:c r="D32" s="51" t="str">
+        <x:v>https://www.nba.com/mavs/mavericks-sign-forward-ray-spalding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33">
+      <x:c r="A33" s="51" t="str">
+        <x:v>S29</x:v>
+      </x:c>
+      <x:c r="B33" s="51" t="str">
+        <x:v>Mavericks — Porzingis trade and Spalding waiver</x:v>
+      </x:c>
+      <x:c r="C33" s="51" t="str">
+        <x:v>Spalding appeared in one Dallas game and was waived in the Jan. 31 roster move</x:v>
+      </x:c>
+      <x:c r="D33" s="51" t="str">
+        <x:v>https://www.nba.com/mavs/mavericks-acquire-all-star-kristaps-porzingis-tim-hardaway-jr-courtney-lee-and-trey-burke-in-trade-with-knicks</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34">
+      <x:c r="A34" s="51" t="str">
+        <x:v>S30</x:v>
+      </x:c>
+      <x:c r="B34" s="51" t="str">
+        <x:v>NBA G League — Ray Spalding</x:v>
+      </x:c>
+      <x:c r="C34" s="51" t="str">
+        <x:v>2018-19 Texas: 29 games, 26 starts, 30.1 MPG</x:v>
+      </x:c>
+      <x:c r="D34" s="51" t="str">
+        <x:v>https://gleague.nba.com/player/1629034/ray-spalding</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="51" t="str">
+        <x:v>S31</x:v>
+      </x:c>
+      <x:c r="B35" s="51" t="str">
+        <x:v>Nuggets — Thomas Welsh two-way</x:v>
+      </x:c>
+      <x:c r="C35" s="51" t="str">
+        <x:v>Denver signed the actual #58 pick to a two-way contract</x:v>
+      </x:c>
+      <x:c r="D35" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/thomas-welsh-signs-two-way-contract-071918</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="51" t="str">
+        <x:v>S32</x:v>
+      </x:c>
+      <x:c r="B36" s="51" t="str">
+        <x:v>Nuggets — 2018-19 two-way preview</x:v>
+      </x:c>
+      <x:c r="C36" s="51" t="str">
+        <x:v>Welsh and Akoon-Purcell occupied Denver's two two-way positions</x:v>
+      </x:c>
+      <x:c r="D36" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/1819-player-previews-akoon-purcell-welsh-091918</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="51" t="str">
+        <x:v>S33</x:v>
+      </x:c>
+      <x:c r="B37" s="51" t="str">
+        <x:v>NBA G League — 2018 two-way rule</x:v>
+      </x:c>
+      <x:c r="C37" s="51" t="str">
+        <x:v>2018-19 teams could carry two two-way players beyond the 15-man roster</x:v>
+      </x:c>
+      <x:c r="D37" s="51" t="str">
+        <x:v>https://windycity.gleague.nba.com/news/bulls-sign-brandon-sampson-to-two-way-contract</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="51" t="str">
+        <x:v>S34</x:v>
+      </x:c>
+      <x:c r="B38" s="51" t="str">
+        <x:v>Nuggets — Welsh 2018-19 recap</x:v>
+      </x:c>
+      <x:c r="C38" s="51" t="str">
+        <x:v>Welsh played 11 NBA games and 36 minutes; G League was his primary venue</x:v>
+      </x:c>
+      <x:c r="D38" s="51" t="str">
+        <x:v>https://www.nba.com/nuggets/news/denver-nuggets-thomas-welsh-excited-for-nba-summer-league-070219c</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="51" t="str">
+        <x:v>S35</x:v>
+      </x:c>
+      <x:c r="B39" s="51" t="str">
+        <x:v>RealGM — Thomas Welsh profile</x:v>
+      </x:c>
+      <x:c r="C39" s="51" t="str">
+        <x:v>Two-way transaction and 20-game G League allocation baseline</x:v>
+      </x:c>
+      <x:c r="D39" s="51" t="str">
+        <x:v>https://basketball.realgm.com/player/Thomas-Welsh/Summary/64323</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="51" t="str">
+        <x:v>S36</x:v>
+      </x:c>
+      <x:c r="B40" s="51" t="str">
+        <x:v>NBA — 2018-11-15 Atlanta at Denver</x:v>
+      </x:c>
+      <x:c r="C40" s="51" t="str">
+        <x:v>Denver 138-93 official game baseline</x:v>
+      </x:c>
+      <x:c r="D40" s="51" t="str">
+        <x:v>https://www.nba.com/game/atl-vs-den-0021800214</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="41">
+      <x:c r="A41" s="51" t="str">
+        <x:v>S37</x:v>
+      </x:c>
+      <x:c r="B41" s="51" t="str">
+        <x:v>Basketball-Reference — 2018-11-15 box score</x:v>
+      </x:c>
+      <x:c r="C41" s="51" t="str">
+        <x:v>Welsh did not play against Atlanta</x:v>
+      </x:c>
+      <x:c r="D41" s="51" t="str">
+        <x:v>https://www.basketball-reference.com/boxscores/201811150DEN.html</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="42">
+      <x:c r="A42" s="51" t="str">
+        <x:v>S38</x:v>
+      </x:c>
+      <x:c r="B42" s="51" t="str">
+        <x:v>NBA Hawks — 2018-12-08 Denver at Atlanta</x:v>
+      </x:c>
+      <x:c r="C42" s="51" t="str">
+        <x:v>Atlanta 106-98 official game baseline</x:v>
+      </x:c>
+      <x:c r="D42" s="51" t="str">
+        <x:v>https://www.nba.com/hawks/game/0021800380</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="51" t="str">
+        <x:v>S39</x:v>
+      </x:c>
+      <x:c r="B43" s="51" t="str">
+        <x:v>Basketball-Reference — 2018-12-08 box score</x:v>
+      </x:c>
+      <x:c r="C43" s="51" t="str">
+        <x:v>Welsh did not play against Atlanta</x:v>
+      </x:c>
+      <x:c r="D43" s="51" t="str">
+        <x:v>https://www.basketball-reference.com/boxscores/201812080ATL.html</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12185,7 +13163,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R31c25f5cf78044f3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52b7422b3c84448d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>